<commit_message>
Implementacion de login, logout y register con sus views
</commit_message>
<xml_diff>
--- a/diagramaGANTT.xlsx
+++ b/diagramaGANTT.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8EFBE45-23E5-4395-9AAE-EA6F918A6D78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE96ECD3-F529-4E6D-874A-E8FFF83967B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1208,6 +1208,30 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="44" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="44" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="44" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="44" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="45" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="45" borderId="2" xfId="12" applyFill="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="45" borderId="2" xfId="10" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="169" fontId="0" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -1219,30 +1243,6 @@
     </xf>
     <xf numFmtId="168" fontId="6" fillId="0" borderId="3" xfId="9" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="44" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="44" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="44" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="44" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="45" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="45" borderId="2" xfId="12" applyFill="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="45" borderId="2" xfId="10" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="54">
@@ -1929,11 +1929,10 @@
         <v>4</v>
       </c>
       <c r="C3" s="52"/>
-      <c r="D3" s="60">
-        <f ca="1">TODAY()</f>
+      <c r="D3" s="68">
         <v>46113</v>
       </c>
-      <c r="E3" s="60"/>
+      <c r="E3" s="68"/>
     </row>
     <row r="4" spans="1:63" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="26" t="s">
@@ -1943,86 +1942,86 @@
       <c r="D4" s="5">
         <v>1</v>
       </c>
-      <c r="H4" s="57">
-        <f ca="1">H5</f>
+      <c r="H4" s="65">
+        <f>H5</f>
         <v>46111</v>
       </c>
-      <c r="I4" s="58"/>
-      <c r="J4" s="58"/>
-      <c r="K4" s="58"/>
-      <c r="L4" s="58"/>
-      <c r="M4" s="58"/>
-      <c r="N4" s="59"/>
-      <c r="O4" s="57">
-        <f ca="1">O5</f>
+      <c r="I4" s="66"/>
+      <c r="J4" s="66"/>
+      <c r="K4" s="66"/>
+      <c r="L4" s="66"/>
+      <c r="M4" s="66"/>
+      <c r="N4" s="67"/>
+      <c r="O4" s="65">
+        <f>O5</f>
         <v>46118</v>
       </c>
-      <c r="P4" s="58"/>
-      <c r="Q4" s="58"/>
-      <c r="R4" s="58"/>
-      <c r="S4" s="58"/>
-      <c r="T4" s="58"/>
-      <c r="U4" s="59"/>
-      <c r="V4" s="57">
-        <f ca="1">V5</f>
+      <c r="P4" s="66"/>
+      <c r="Q4" s="66"/>
+      <c r="R4" s="66"/>
+      <c r="S4" s="66"/>
+      <c r="T4" s="66"/>
+      <c r="U4" s="67"/>
+      <c r="V4" s="65">
+        <f>V5</f>
         <v>46125</v>
       </c>
-      <c r="W4" s="58"/>
-      <c r="X4" s="58"/>
-      <c r="Y4" s="58"/>
-      <c r="Z4" s="58"/>
-      <c r="AA4" s="58"/>
-      <c r="AB4" s="59"/>
-      <c r="AC4" s="57">
-        <f ca="1">AC5</f>
+      <c r="W4" s="66"/>
+      <c r="X4" s="66"/>
+      <c r="Y4" s="66"/>
+      <c r="Z4" s="66"/>
+      <c r="AA4" s="66"/>
+      <c r="AB4" s="67"/>
+      <c r="AC4" s="65">
+        <f>AC5</f>
         <v>46132</v>
       </c>
-      <c r="AD4" s="58"/>
-      <c r="AE4" s="58"/>
-      <c r="AF4" s="58"/>
-      <c r="AG4" s="58"/>
-      <c r="AH4" s="58"/>
-      <c r="AI4" s="59"/>
-      <c r="AJ4" s="57">
-        <f ca="1">AJ5</f>
+      <c r="AD4" s="66"/>
+      <c r="AE4" s="66"/>
+      <c r="AF4" s="66"/>
+      <c r="AG4" s="66"/>
+      <c r="AH4" s="66"/>
+      <c r="AI4" s="67"/>
+      <c r="AJ4" s="65">
+        <f>AJ5</f>
         <v>46139</v>
       </c>
-      <c r="AK4" s="58"/>
-      <c r="AL4" s="58"/>
-      <c r="AM4" s="58"/>
-      <c r="AN4" s="58"/>
-      <c r="AO4" s="58"/>
-      <c r="AP4" s="59"/>
-      <c r="AQ4" s="57">
-        <f ca="1">AQ5</f>
+      <c r="AK4" s="66"/>
+      <c r="AL4" s="66"/>
+      <c r="AM4" s="66"/>
+      <c r="AN4" s="66"/>
+      <c r="AO4" s="66"/>
+      <c r="AP4" s="67"/>
+      <c r="AQ4" s="65">
+        <f>AQ5</f>
         <v>46146</v>
       </c>
-      <c r="AR4" s="58"/>
-      <c r="AS4" s="58"/>
-      <c r="AT4" s="58"/>
-      <c r="AU4" s="58"/>
-      <c r="AV4" s="58"/>
-      <c r="AW4" s="59"/>
-      <c r="AX4" s="57">
-        <f ca="1">AX5</f>
+      <c r="AR4" s="66"/>
+      <c r="AS4" s="66"/>
+      <c r="AT4" s="66"/>
+      <c r="AU4" s="66"/>
+      <c r="AV4" s="66"/>
+      <c r="AW4" s="67"/>
+      <c r="AX4" s="65">
+        <f>AX5</f>
         <v>46153</v>
       </c>
-      <c r="AY4" s="58"/>
-      <c r="AZ4" s="58"/>
-      <c r="BA4" s="58"/>
-      <c r="BB4" s="58"/>
-      <c r="BC4" s="58"/>
-      <c r="BD4" s="59"/>
-      <c r="BE4" s="57">
-        <f ca="1">BE5</f>
+      <c r="AY4" s="66"/>
+      <c r="AZ4" s="66"/>
+      <c r="BA4" s="66"/>
+      <c r="BB4" s="66"/>
+      <c r="BC4" s="66"/>
+      <c r="BD4" s="67"/>
+      <c r="BE4" s="65">
+        <f>BE5</f>
         <v>46160</v>
       </c>
-      <c r="BF4" s="58"/>
-      <c r="BG4" s="58"/>
-      <c r="BH4" s="58"/>
-      <c r="BI4" s="58"/>
-      <c r="BJ4" s="58"/>
-      <c r="BK4" s="59"/>
+      <c r="BF4" s="66"/>
+      <c r="BG4" s="66"/>
+      <c r="BH4" s="66"/>
+      <c r="BI4" s="66"/>
+      <c r="BJ4" s="66"/>
+      <c r="BK4" s="67"/>
     </row>
     <row r="5" spans="1:63" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="26" t="s">
@@ -2034,227 +2033,227 @@
       <c r="E5" s="34"/>
       <c r="F5" s="34"/>
       <c r="H5" s="49">
-        <f ca="1">Inicio_del_proyecto-WEEKDAY(Inicio_del_proyecto,1)+2+7*(Semana_para_mostrar-1)</f>
+        <f>Inicio_del_proyecto-WEEKDAY(Inicio_del_proyecto,1)+2+7*(Semana_para_mostrar-1)</f>
         <v>46111</v>
       </c>
       <c r="I5" s="50">
-        <f ca="1">H5+1</f>
+        <f>H5+1</f>
         <v>46112</v>
       </c>
       <c r="J5" s="50">
-        <f ca="1">I5+1</f>
+        <f>I5+1</f>
         <v>46113</v>
       </c>
       <c r="K5" s="50">
-        <f t="shared" ref="K5:AW5" ca="1" si="0">J5+1</f>
+        <f t="shared" ref="K5:AW5" si="0">J5+1</f>
         <v>46114</v>
       </c>
       <c r="L5" s="50">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>46115</v>
       </c>
       <c r="M5" s="50">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>46116</v>
       </c>
       <c r="N5" s="51">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>46117</v>
       </c>
       <c r="O5" s="49">
-        <f ca="1">N5+1</f>
+        <f>N5+1</f>
         <v>46118</v>
       </c>
       <c r="P5" s="50">
-        <f ca="1">O5+1</f>
+        <f>O5+1</f>
         <v>46119</v>
       </c>
       <c r="Q5" s="50">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>46120</v>
       </c>
       <c r="R5" s="50">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>46121</v>
       </c>
       <c r="S5" s="50">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>46122</v>
       </c>
       <c r="T5" s="50">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>46123</v>
       </c>
       <c r="U5" s="51">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>46124</v>
       </c>
       <c r="V5" s="49">
-        <f ca="1">U5+1</f>
+        <f>U5+1</f>
         <v>46125</v>
       </c>
       <c r="W5" s="50">
-        <f ca="1">V5+1</f>
+        <f>V5+1</f>
         <v>46126</v>
       </c>
       <c r="X5" s="50">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>46127</v>
       </c>
       <c r="Y5" s="50">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>46128</v>
       </c>
       <c r="Z5" s="50">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>46129</v>
       </c>
       <c r="AA5" s="50">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>46130</v>
       </c>
       <c r="AB5" s="51">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>46131</v>
       </c>
       <c r="AC5" s="49">
-        <f ca="1">AB5+1</f>
+        <f>AB5+1</f>
         <v>46132</v>
       </c>
       <c r="AD5" s="50">
-        <f ca="1">AC5+1</f>
+        <f>AC5+1</f>
         <v>46133</v>
       </c>
       <c r="AE5" s="50">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>46134</v>
       </c>
       <c r="AF5" s="50">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>46135</v>
       </c>
       <c r="AG5" s="50">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>46136</v>
       </c>
       <c r="AH5" s="50">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>46137</v>
       </c>
       <c r="AI5" s="51">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>46138</v>
       </c>
       <c r="AJ5" s="49">
-        <f ca="1">AI5+1</f>
+        <f>AI5+1</f>
         <v>46139</v>
       </c>
       <c r="AK5" s="50">
-        <f ca="1">AJ5+1</f>
+        <f>AJ5+1</f>
         <v>46140</v>
       </c>
       <c r="AL5" s="50">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>46141</v>
       </c>
       <c r="AM5" s="50">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>46142</v>
       </c>
       <c r="AN5" s="50">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>46143</v>
       </c>
       <c r="AO5" s="50">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>46144</v>
       </c>
       <c r="AP5" s="51">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>46145</v>
       </c>
       <c r="AQ5" s="49">
-        <f ca="1">AP5+1</f>
+        <f>AP5+1</f>
         <v>46146</v>
       </c>
       <c r="AR5" s="50">
-        <f ca="1">AQ5+1</f>
+        <f>AQ5+1</f>
         <v>46147</v>
       </c>
       <c r="AS5" s="50">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>46148</v>
       </c>
       <c r="AT5" s="50">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>46149</v>
       </c>
       <c r="AU5" s="50">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>46150</v>
       </c>
       <c r="AV5" s="50">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>46151</v>
       </c>
       <c r="AW5" s="51">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>46152</v>
       </c>
       <c r="AX5" s="49">
-        <f ca="1">AW5+1</f>
+        <f>AW5+1</f>
         <v>46153</v>
       </c>
       <c r="AY5" s="50">
-        <f ca="1">AX5+1</f>
+        <f>AX5+1</f>
         <v>46154</v>
       </c>
       <c r="AZ5" s="50">
-        <f t="shared" ref="AZ5:BD5" ca="1" si="1">AY5+1</f>
+        <f t="shared" ref="AZ5:BD5" si="1">AY5+1</f>
         <v>46155</v>
       </c>
       <c r="BA5" s="50">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>46156</v>
       </c>
       <c r="BB5" s="50">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>46157</v>
       </c>
       <c r="BC5" s="50">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>46158</v>
       </c>
       <c r="BD5" s="51">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>46159</v>
       </c>
       <c r="BE5" s="49">
-        <f ca="1">BD5+1</f>
+        <f>BD5+1</f>
         <v>46160</v>
       </c>
       <c r="BF5" s="50">
-        <f ca="1">BE5+1</f>
+        <f>BE5+1</f>
         <v>46161</v>
       </c>
       <c r="BG5" s="50">
-        <f t="shared" ref="BG5:BK5" ca="1" si="2">BF5+1</f>
+        <f t="shared" ref="BG5:BK5" si="2">BF5+1</f>
         <v>46162</v>
       </c>
       <c r="BH5" s="50">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>46163</v>
       </c>
       <c r="BI5" s="50">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>46164</v>
       </c>
       <c r="BJ5" s="50">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>46165</v>
       </c>
       <c r="BK5" s="51">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>46166</v>
       </c>
     </row>
@@ -2279,227 +2278,227 @@
         <v>12</v>
       </c>
       <c r="H6" s="8" t="str">
-        <f t="shared" ref="H6" ca="1" si="3">LEFT(TEXT(H5,"ddd"),1)</f>
+        <f t="shared" ref="H6" si="3">LEFT(TEXT(H5,"ddd"),1)</f>
         <v>l</v>
       </c>
       <c r="I6" s="8" t="str">
-        <f t="shared" ref="I6:AQ6" ca="1" si="4">LEFT(TEXT(I5,"ddd"),1)</f>
+        <f t="shared" ref="I6:AQ6" si="4">LEFT(TEXT(I5,"ddd"),1)</f>
         <v>m</v>
       </c>
       <c r="J6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>m</v>
       </c>
       <c r="K6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>j</v>
       </c>
       <c r="L6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>v</v>
       </c>
       <c r="M6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>s</v>
       </c>
       <c r="N6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>d</v>
       </c>
       <c r="O6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>l</v>
       </c>
       <c r="P6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>m</v>
       </c>
       <c r="Q6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>m</v>
       </c>
       <c r="R6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>j</v>
       </c>
       <c r="S6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>v</v>
       </c>
       <c r="T6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>s</v>
       </c>
       <c r="U6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>d</v>
       </c>
       <c r="V6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>l</v>
       </c>
       <c r="W6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>m</v>
       </c>
       <c r="X6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>m</v>
       </c>
       <c r="Y6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>j</v>
       </c>
       <c r="Z6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>v</v>
       </c>
       <c r="AA6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>s</v>
       </c>
       <c r="AB6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>d</v>
       </c>
       <c r="AC6" s="8" t="str">
-        <f ca="1">LEFT(TEXT(AC5,"ddd"),1)</f>
+        <f>LEFT(TEXT(AC5,"ddd"),1)</f>
         <v>l</v>
       </c>
       <c r="AD6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>m</v>
       </c>
       <c r="AE6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>m</v>
       </c>
       <c r="AF6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>j</v>
       </c>
       <c r="AG6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>v</v>
       </c>
       <c r="AH6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>s</v>
       </c>
       <c r="AI6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>d</v>
       </c>
       <c r="AJ6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>l</v>
       </c>
       <c r="AK6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>m</v>
       </c>
       <c r="AL6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>m</v>
       </c>
       <c r="AM6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>j</v>
       </c>
       <c r="AN6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>v</v>
       </c>
       <c r="AO6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>s</v>
       </c>
       <c r="AP6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>d</v>
       </c>
       <c r="AQ6" s="8" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>l</v>
       </c>
       <c r="AR6" s="8" t="str">
-        <f t="shared" ref="AR6:CU6" ca="1" si="5">LEFT(TEXT(AR5,"ddd"),1)</f>
+        <f t="shared" ref="AR6:BK6" si="5">LEFT(TEXT(AR5,"ddd"),1)</f>
         <v>m</v>
       </c>
       <c r="AS6" s="8" t="str">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" si="5"/>
         <v>m</v>
       </c>
       <c r="AT6" s="8" t="str">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" si="5"/>
         <v>j</v>
       </c>
       <c r="AU6" s="8" t="str">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" si="5"/>
         <v>v</v>
       </c>
       <c r="AV6" s="8" t="str">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" si="5"/>
         <v>s</v>
       </c>
       <c r="AW6" s="8" t="str">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" si="5"/>
         <v>d</v>
       </c>
       <c r="AX6" s="8" t="str">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" si="5"/>
         <v>l</v>
       </c>
       <c r="AY6" s="8" t="str">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" si="5"/>
         <v>m</v>
       </c>
       <c r="AZ6" s="8" t="str">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" si="5"/>
         <v>m</v>
       </c>
       <c r="BA6" s="8" t="str">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" si="5"/>
         <v>j</v>
       </c>
       <c r="BB6" s="8" t="str">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" si="5"/>
         <v>v</v>
       </c>
       <c r="BC6" s="8" t="str">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" si="5"/>
         <v>s</v>
       </c>
       <c r="BD6" s="8" t="str">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" si="5"/>
         <v>d</v>
       </c>
       <c r="BE6" s="8" t="str">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" si="5"/>
         <v>l</v>
       </c>
       <c r="BF6" s="8" t="str">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" si="5"/>
         <v>m</v>
       </c>
       <c r="BG6" s="8" t="str">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" si="5"/>
         <v>m</v>
       </c>
       <c r="BH6" s="8" t="str">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" si="5"/>
         <v>j</v>
       </c>
       <c r="BI6" s="8" t="str">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" si="5"/>
         <v>v</v>
       </c>
       <c r="BJ6" s="8" t="str">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" si="5"/>
         <v>s</v>
       </c>
       <c r="BK6" s="8" t="str">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" si="5"/>
         <v>d</v>
       </c>
     </row>
@@ -2633,7 +2632,7 @@
       <c r="BB8" s="22"/>
       <c r="BC8" s="22"/>
       <c r="BD8" s="22"/>
-      <c r="BE8" s="68"/>
+      <c r="BE8" s="64"/>
       <c r="BF8" s="22"/>
       <c r="BG8" s="22"/>
       <c r="BH8" s="22"/>
@@ -2652,16 +2651,16 @@
         <v>1</v>
       </c>
       <c r="D9" s="39">
-        <f ca="1">Inicio_del_proyecto</f>
+        <f>Inicio_del_proyecto</f>
         <v>46113</v>
       </c>
       <c r="E9" s="39">
-        <f ca="1">D9</f>
+        <f>D9</f>
         <v>46113</v>
       </c>
       <c r="F9" s="9"/>
       <c r="G9" s="9">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="H9" s="22"/>
@@ -2732,16 +2731,16 @@
         <v>1</v>
       </c>
       <c r="D10" s="39">
-        <f ca="1">E9</f>
+        <f>E9</f>
         <v>46113</v>
       </c>
       <c r="E10" s="39">
-        <f ca="1">D10</f>
+        <f>D10</f>
         <v>46113</v>
       </c>
       <c r="F10" s="9"/>
       <c r="G10" s="9">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="H10" s="22"/>
@@ -2810,16 +2809,16 @@
         <v>0.9</v>
       </c>
       <c r="D11" s="39">
-        <f ca="1">E10+1</f>
+        <f>E10+1</f>
         <v>46114</v>
       </c>
       <c r="E11" s="39">
-        <f ca="1">D11</f>
+        <f>D11</f>
         <v>46114</v>
       </c>
       <c r="F11" s="9"/>
       <c r="G11" s="9">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="H11" s="22"/>
@@ -2956,19 +2955,19 @@
         <v>26</v>
       </c>
       <c r="C13" s="15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D13" s="42">
-        <f ca="1">E11+1</f>
+        <f>E11+1</f>
         <v>46115</v>
       </c>
       <c r="E13" s="42">
-        <f ca="1">D13+1</f>
+        <f>D13+1</f>
         <v>46116</v>
       </c>
       <c r="F13" s="9"/>
       <c r="G13" s="9">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="H13" s="22"/>
@@ -3034,19 +3033,19 @@
         <v>27</v>
       </c>
       <c r="C14" s="15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D14" s="42">
-        <f t="shared" ref="D14:D28" ca="1" si="7">E13+1</f>
+        <f t="shared" ref="D14:D28" si="7">E13+1</f>
         <v>46117</v>
       </c>
       <c r="E14" s="42">
-        <f ca="1">D14+1</f>
+        <f>D14+1</f>
         <v>46118</v>
       </c>
       <c r="F14" s="9"/>
       <c r="G14" s="9">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="H14" s="22"/>
@@ -3112,19 +3111,19 @@
         <v>28</v>
       </c>
       <c r="C15" s="15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D15" s="42">
-        <f t="shared" ca="1" si="7"/>
+        <f t="shared" si="7"/>
         <v>46119</v>
       </c>
       <c r="E15" s="42">
-        <f ca="1">D15</f>
+        <f>D15</f>
         <v>46119</v>
       </c>
       <c r="F15" s="9"/>
       <c r="G15" s="9">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="H15" s="22"/>
@@ -3187,20 +3186,22 @@
     <row r="16" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="25"/>
       <c r="B16" s="31" t="s">
-        <v>29</v>
-      </c>
-      <c r="C16" s="15"/>
+        <v>30</v>
+      </c>
+      <c r="C16" s="15">
+        <v>1</v>
+      </c>
       <c r="D16" s="42">
-        <f t="shared" ca="1" si="7"/>
-        <v>46120</v>
+        <f>E15</f>
+        <v>46119</v>
       </c>
       <c r="E16" s="42">
-        <f ca="1">D16</f>
-        <v>46120</v>
+        <f>D16</f>
+        <v>46119</v>
       </c>
       <c r="F16" s="9"/>
       <c r="G16" s="9">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="H16" s="22"/>
@@ -3263,20 +3264,20 @@
     <row r="17" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="25"/>
       <c r="B17" s="31" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C17" s="15"/>
       <c r="D17" s="42">
-        <f t="shared" ca="1" si="7"/>
-        <v>46121</v>
+        <f t="shared" si="7"/>
+        <v>46120</v>
       </c>
       <c r="E17" s="42">
-        <f ca="1">D17</f>
-        <v>46121</v>
+        <f>D17</f>
+        <v>46120</v>
       </c>
       <c r="F17" s="9"/>
       <c r="G17" s="9">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="H17" s="22"/>
@@ -3343,16 +3344,16 @@
       </c>
       <c r="C18" s="15"/>
       <c r="D18" s="42">
-        <f t="shared" ca="1" si="7"/>
-        <v>46122</v>
+        <f t="shared" si="7"/>
+        <v>46121</v>
       </c>
       <c r="E18" s="42">
-        <f ca="1">D18+2</f>
-        <v>46124</v>
+        <f>D18+2</f>
+        <v>46123</v>
       </c>
       <c r="F18" s="9"/>
       <c r="G18" s="9">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>3</v>
       </c>
       <c r="H18" s="22"/>
@@ -3419,12 +3420,12 @@
       </c>
       <c r="C19" s="15"/>
       <c r="D19" s="42">
-        <f t="shared" ca="1" si="7"/>
-        <v>46125</v>
+        <f t="shared" si="7"/>
+        <v>46124</v>
       </c>
       <c r="E19" s="42">
-        <f ca="1">D19+2</f>
-        <v>46127</v>
+        <f>D19+2</f>
+        <v>46126</v>
       </c>
       <c r="F19" s="9"/>
       <c r="G19" s="9"/>
@@ -3492,12 +3493,12 @@
       </c>
       <c r="C20" s="15"/>
       <c r="D20" s="42">
-        <f t="shared" ca="1" si="7"/>
+        <f t="shared" si="7"/>
+        <v>46127</v>
+      </c>
+      <c r="E20" s="42">
+        <f>D20+1</f>
         <v>46128</v>
-      </c>
-      <c r="E20" s="42">
-        <f ca="1">D20+1</f>
-        <v>46129</v>
       </c>
       <c r="F20" s="9"/>
       <c r="G20" s="9"/>
@@ -3565,12 +3566,12 @@
       </c>
       <c r="C21" s="15"/>
       <c r="D21" s="42">
-        <f t="shared" ca="1" si="7"/>
+        <f t="shared" si="7"/>
+        <v>46129</v>
+      </c>
+      <c r="E21" s="42">
+        <f>D21+1</f>
         <v>46130</v>
-      </c>
-      <c r="E21" s="42">
-        <f ca="1">D21+1</f>
-        <v>46131</v>
       </c>
       <c r="F21" s="9"/>
       <c r="G21" s="9"/>
@@ -3638,12 +3639,12 @@
       </c>
       <c r="C22" s="15"/>
       <c r="D22" s="42">
-        <f t="shared" ca="1" si="7"/>
-        <v>46132</v>
+        <f t="shared" si="7"/>
+        <v>46131</v>
       </c>
       <c r="E22" s="42">
-        <f ca="1">D22</f>
-        <v>46132</v>
+        <f>D22</f>
+        <v>46131</v>
       </c>
       <c r="F22" s="9"/>
       <c r="G22" s="9"/>
@@ -3711,12 +3712,12 @@
       </c>
       <c r="C23" s="15"/>
       <c r="D23" s="42">
-        <f t="shared" ca="1" si="7"/>
-        <v>46133</v>
+        <f t="shared" si="7"/>
+        <v>46132</v>
       </c>
       <c r="E23" s="42">
-        <f ca="1">D23+2</f>
-        <v>46135</v>
+        <f>D23+2</f>
+        <v>46134</v>
       </c>
       <c r="F23" s="9"/>
       <c r="G23" s="9"/>
@@ -3784,12 +3785,12 @@
       </c>
       <c r="C24" s="15"/>
       <c r="D24" s="42">
-        <f t="shared" ca="1" si="7"/>
+        <f t="shared" si="7"/>
+        <v>46135</v>
+      </c>
+      <c r="E24" s="42">
+        <f>D24+1</f>
         <v>46136</v>
-      </c>
-      <c r="E24" s="42">
-        <f ca="1">D24+1</f>
-        <v>46137</v>
       </c>
       <c r="F24" s="9"/>
       <c r="G24" s="9"/>
@@ -3857,12 +3858,12 @@
       </c>
       <c r="C25" s="15"/>
       <c r="D25" s="42">
-        <f t="shared" ca="1" si="7"/>
+        <f t="shared" si="7"/>
+        <v>46137</v>
+      </c>
+      <c r="E25" s="42">
+        <f>D25+1</f>
         <v>46138</v>
-      </c>
-      <c r="E25" s="42">
-        <f ca="1">D25+1</f>
-        <v>46139</v>
       </c>
       <c r="F25" s="9"/>
       <c r="G25" s="9"/>
@@ -3930,12 +3931,12 @@
       </c>
       <c r="C26" s="15"/>
       <c r="D26" s="42">
-        <f t="shared" ca="1" si="7"/>
+        <f t="shared" si="7"/>
+        <v>46139</v>
+      </c>
+      <c r="E26" s="42">
+        <f>D26+1</f>
         <v>46140</v>
-      </c>
-      <c r="E26" s="42">
-        <f ca="1">D26+1</f>
-        <v>46141</v>
       </c>
       <c r="F26" s="9"/>
       <c r="G26" s="9"/>
@@ -4003,12 +4004,12 @@
       </c>
       <c r="C27" s="15"/>
       <c r="D27" s="42">
-        <f t="shared" ca="1" si="7"/>
-        <v>46142</v>
+        <f t="shared" si="7"/>
+        <v>46141</v>
       </c>
       <c r="E27" s="42">
-        <f ca="1">D27+2</f>
-        <v>46144</v>
+        <f>D27+2</f>
+        <v>46143</v>
       </c>
       <c r="F27" s="9"/>
       <c r="G27" s="9"/>
@@ -4076,12 +4077,12 @@
       </c>
       <c r="C28" s="15"/>
       <c r="D28" s="42">
-        <f t="shared" ca="1" si="7"/>
-        <v>46145</v>
+        <f t="shared" si="7"/>
+        <v>46144</v>
       </c>
       <c r="E28" s="42">
-        <f ca="1">D28+2</f>
-        <v>46147</v>
+        <f>D28+2</f>
+        <v>46146</v>
       </c>
       <c r="F28" s="9"/>
       <c r="G28" s="9"/>
@@ -4221,16 +4222,16 @@
       </c>
       <c r="C30" s="18"/>
       <c r="D30" s="45">
-        <f ca="1">E28+1</f>
+        <f>E28+1</f>
+        <v>46147</v>
+      </c>
+      <c r="E30" s="45">
+        <f t="shared" ref="E30:E40" si="8">D30+1</f>
         <v>46148</v>
-      </c>
-      <c r="E30" s="45">
-        <f ca="1">D30+1</f>
-        <v>46149</v>
       </c>
       <c r="F30" s="9"/>
       <c r="G30" s="9">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="H30" s="22"/>
@@ -4297,16 +4298,16 @@
       </c>
       <c r="C31" s="18"/>
       <c r="D31" s="45">
-        <f ca="1">D30</f>
+        <f>D30</f>
+        <v>46147</v>
+      </c>
+      <c r="E31" s="45">
+        <f t="shared" si="8"/>
         <v>46148</v>
-      </c>
-      <c r="E31" s="45">
-        <f ca="1">D31+1</f>
-        <v>46149</v>
       </c>
       <c r="F31" s="9"/>
       <c r="G31" s="9">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="H31" s="22"/>
@@ -4373,16 +4374,16 @@
       </c>
       <c r="C32" s="18"/>
       <c r="D32" s="45">
-        <f ca="1">D31</f>
+        <f>D31</f>
+        <v>46147</v>
+      </c>
+      <c r="E32" s="45">
+        <f t="shared" si="8"/>
         <v>46148</v>
-      </c>
-      <c r="E32" s="45">
-        <f ca="1">D32+1</f>
-        <v>46149</v>
       </c>
       <c r="F32" s="9"/>
       <c r="G32" s="9">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="H32" s="22"/>
@@ -4449,16 +4450,16 @@
       </c>
       <c r="C33" s="18"/>
       <c r="D33" s="45">
-        <f ca="1">D32</f>
+        <f>D32</f>
+        <v>46147</v>
+      </c>
+      <c r="E33" s="45">
+        <f t="shared" si="8"/>
         <v>46148</v>
-      </c>
-      <c r="E33" s="45">
-        <f ca="1">D33+1</f>
-        <v>46149</v>
       </c>
       <c r="F33" s="9"/>
       <c r="G33" s="9">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="H33" s="22"/>
@@ -4525,16 +4526,16 @@
       </c>
       <c r="C34" s="18"/>
       <c r="D34" s="45">
-        <f ca="1">D33</f>
+        <f>D33</f>
+        <v>46147</v>
+      </c>
+      <c r="E34" s="45">
+        <f t="shared" si="8"/>
         <v>46148</v>
-      </c>
-      <c r="E34" s="45">
-        <f ca="1">D34+1</f>
-        <v>46149</v>
       </c>
       <c r="F34" s="9"/>
       <c r="G34" s="9">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="H34" s="22"/>
@@ -4601,12 +4602,12 @@
       </c>
       <c r="C35" s="18"/>
       <c r="D35" s="45">
-        <f ca="1">E34+1</f>
+        <f>E34+1</f>
+        <v>46149</v>
+      </c>
+      <c r="E35" s="45">
+        <f t="shared" si="8"/>
         <v>46150</v>
-      </c>
-      <c r="E35" s="45">
-        <f ca="1">D35+1</f>
-        <v>46151</v>
       </c>
       <c r="F35" s="9"/>
       <c r="G35" s="9"/>
@@ -4674,12 +4675,12 @@
       </c>
       <c r="C36" s="18"/>
       <c r="D36" s="45">
-        <f ca="1">D35</f>
+        <f>D35</f>
+        <v>46149</v>
+      </c>
+      <c r="E36" s="45">
+        <f t="shared" si="8"/>
         <v>46150</v>
-      </c>
-      <c r="E36" s="45">
-        <f ca="1">D36+1</f>
-        <v>46151</v>
       </c>
       <c r="F36" s="9"/>
       <c r="G36" s="9"/>
@@ -4747,12 +4748,12 @@
       </c>
       <c r="C37" s="18"/>
       <c r="D37" s="45">
-        <f ca="1">D36</f>
+        <f>D36</f>
+        <v>46149</v>
+      </c>
+      <c r="E37" s="45">
+        <f t="shared" si="8"/>
         <v>46150</v>
-      </c>
-      <c r="E37" s="45">
-        <f ca="1">D37+1</f>
-        <v>46151</v>
       </c>
       <c r="F37" s="9"/>
       <c r="G37" s="9"/>
@@ -4820,12 +4821,12 @@
       </c>
       <c r="C38" s="18"/>
       <c r="D38" s="45">
-        <f ca="1">D37</f>
+        <f>D37</f>
+        <v>46149</v>
+      </c>
+      <c r="E38" s="45">
+        <f t="shared" si="8"/>
         <v>46150</v>
-      </c>
-      <c r="E38" s="45">
-        <f ca="1">D38+1</f>
-        <v>46151</v>
       </c>
       <c r="F38" s="9"/>
       <c r="G38" s="9"/>
@@ -4893,12 +4894,12 @@
       </c>
       <c r="C39" s="18"/>
       <c r="D39" s="45">
-        <f ca="1">D38</f>
+        <f>D38</f>
+        <v>46149</v>
+      </c>
+      <c r="E39" s="45">
+        <f t="shared" si="8"/>
         <v>46150</v>
-      </c>
-      <c r="E39" s="45">
-        <f ca="1">D39+1</f>
-        <v>46151</v>
       </c>
       <c r="F39" s="9"/>
       <c r="G39" s="9"/>
@@ -4966,12 +4967,12 @@
       </c>
       <c r="C40" s="18"/>
       <c r="D40" s="45">
-        <f ca="1">E39+1</f>
+        <f>E39+1</f>
+        <v>46151</v>
+      </c>
+      <c r="E40" s="45">
+        <f t="shared" si="8"/>
         <v>46152</v>
-      </c>
-      <c r="E40" s="45">
-        <f ca="1">D40+1</f>
-        <v>46153</v>
       </c>
       <c r="F40" s="9"/>
       <c r="G40" s="9"/>
@@ -5111,16 +5112,16 @@
       </c>
       <c r="C42" s="21"/>
       <c r="D42" s="48">
-        <f ca="1">E40+1</f>
-        <v>46154</v>
+        <f>E40+1</f>
+        <v>46153</v>
       </c>
       <c r="E42" s="48">
-        <f ca="1">D42</f>
-        <v>46154</v>
+        <f>D42</f>
+        <v>46153</v>
       </c>
       <c r="F42" s="9"/>
       <c r="G42" s="9">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="H42" s="22"/>
@@ -5187,16 +5188,16 @@
       </c>
       <c r="C43" s="21"/>
       <c r="D43" s="48">
-        <f ca="1">E42+1</f>
+        <f>E42+1</f>
+        <v>46154</v>
+      </c>
+      <c r="E43" s="48">
+        <f>D43+1</f>
         <v>46155</v>
-      </c>
-      <c r="E43" s="48">
-        <f ca="1">D43+1</f>
-        <v>46156</v>
       </c>
       <c r="F43" s="9"/>
       <c r="G43" s="9">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="H43" s="22"/>
@@ -5263,16 +5264,16 @@
       </c>
       <c r="C44" s="21"/>
       <c r="D44" s="48">
-        <f ca="1">E43+1</f>
+        <f>E43+1</f>
+        <v>46156</v>
+      </c>
+      <c r="E44" s="48">
+        <f>D44+1</f>
         <v>46157</v>
-      </c>
-      <c r="E44" s="48">
-        <f ca="1">D44+1</f>
-        <v>46158</v>
       </c>
       <c r="F44" s="9"/>
       <c r="G44" s="9">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="H44" s="22"/>
@@ -5339,16 +5340,16 @@
       </c>
       <c r="C45" s="21"/>
       <c r="D45" s="48">
-        <f ca="1">E44+1</f>
+        <f>E44+1</f>
+        <v>46158</v>
+      </c>
+      <c r="E45" s="48">
+        <f>D45+1</f>
         <v>46159</v>
-      </c>
-      <c r="E45" s="48">
-        <f ca="1">D45+1</f>
-        <v>46160</v>
       </c>
       <c r="F45" s="9"/>
       <c r="G45" s="9">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="H45" s="22"/>
@@ -5410,12 +5411,12 @@
     </row>
     <row r="46" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="25"/>
-      <c r="B46" s="61" t="s">
+      <c r="B46" s="57" t="s">
         <v>22</v>
       </c>
-      <c r="C46" s="62"/>
-      <c r="D46" s="63"/>
-      <c r="E46" s="64"/>
+      <c r="C46" s="58"/>
+      <c r="D46" s="59"/>
+      <c r="E46" s="60"/>
       <c r="F46" s="9"/>
       <c r="G46" s="9"/>
       <c r="H46" s="22"/>
@@ -5477,17 +5478,17 @@
     </row>
     <row r="47" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="25"/>
-      <c r="B47" s="66" t="s">
+      <c r="B47" s="62" t="s">
         <v>59</v>
       </c>
-      <c r="C47" s="65"/>
-      <c r="D47" s="67">
-        <f ca="1">E45+1</f>
+      <c r="C47" s="61"/>
+      <c r="D47" s="63">
+        <f>E45+1</f>
+        <v>46160</v>
+      </c>
+      <c r="E47" s="63">
+        <f>D47+1</f>
         <v>46161</v>
-      </c>
-      <c r="E47" s="67">
-        <f ca="1">D47+1</f>
-        <v>46162</v>
       </c>
       <c r="F47" s="9"/>
       <c r="G47" s="9"/>
@@ -5550,17 +5551,17 @@
     </row>
     <row r="48" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="25"/>
-      <c r="B48" s="66" t="s">
+      <c r="B48" s="62" t="s">
         <v>60</v>
       </c>
-      <c r="C48" s="65"/>
-      <c r="D48" s="67">
-        <f ca="1">E47+1</f>
+      <c r="C48" s="61"/>
+      <c r="D48" s="63">
+        <f>E47+1</f>
+        <v>46162</v>
+      </c>
+      <c r="E48" s="63">
+        <f>D48+1</f>
         <v>46163</v>
-      </c>
-      <c r="E48" s="67">
-        <f ca="1">D48+1</f>
-        <v>46164</v>
       </c>
       <c r="F48" s="9"/>
       <c r="G48" s="9"/>
@@ -5623,17 +5624,17 @@
     </row>
     <row r="49" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="25"/>
-      <c r="B49" s="66" t="s">
+      <c r="B49" s="62" t="s">
         <v>61</v>
       </c>
-      <c r="C49" s="65"/>
-      <c r="D49" s="67">
-        <f ca="1">E48+1</f>
+      <c r="C49" s="61"/>
+      <c r="D49" s="63">
+        <f>E48+1</f>
+        <v>46164</v>
+      </c>
+      <c r="E49" s="63">
+        <f>D49+1</f>
         <v>46165</v>
-      </c>
-      <c r="E49" s="67">
-        <f ca="1">D49+1</f>
-        <v>46166</v>
       </c>
       <c r="F49" s="9"/>
       <c r="G49" s="9"/>
@@ -5698,21 +5699,21 @@
       <c r="A50" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="B50" s="66" t="s">
+      <c r="B50" s="62" t="s">
         <v>62</v>
       </c>
-      <c r="C50" s="65"/>
-      <c r="D50" s="67">
-        <f ca="1">E49+1</f>
-        <v>46167</v>
-      </c>
-      <c r="E50" s="67">
-        <f ca="1">D50+3</f>
-        <v>46170</v>
+      <c r="C50" s="61"/>
+      <c r="D50" s="63">
+        <f>E49+1</f>
+        <v>46166</v>
+      </c>
+      <c r="E50" s="63">
+        <f>D50+3</f>
+        <v>46169</v>
       </c>
       <c r="F50" s="9"/>
       <c r="G50" s="9">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>4</v>
       </c>
       <c r="H50" s="22"/>
@@ -6437,35 +6438,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Image>
-    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
-    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </ImageTagsTaxHTField>
-    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
-    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="24" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2d714a3296df14eba7a100bb665443ca">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="49549bf45bfbbfb6cffed527380e77e1" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -6753,27 +6725,36 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5144944C-1F1D-4162-962A-96F3FC8455D8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8FE8ED85-58B3-4608-8E91-0433556D50CE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Image>
+    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
+    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </ImageTagsTaxHTField>
+    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
+    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{708DBB9E-6D89-4A94-9DC5-964B7833E11C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6792,4 +6773,24 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8FE8ED85-58B3-4608-8E91-0433556D50CE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5144944C-1F1D-4162-962A-96F3FC8455D8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
+    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizar auth, rutas y configuracion para nuevo catalogo y admin
</commit_message>
<xml_diff>
--- a/diagramaGANTT.xlsx
+++ b/diagramaGANTT.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{279BC165-EBCE-4C78-A0F8-3B310099865E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12AC9A70-4E22-4DB7-AC1D-119728C8EC2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2806,7 +2806,7 @@
         <v>25</v>
       </c>
       <c r="C11" s="12">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="D11" s="39">
         <f>E10+1</f>
@@ -3266,7 +3266,9 @@
       <c r="B17" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="C17" s="15"/>
+      <c r="C17" s="15">
+        <v>1</v>
+      </c>
       <c r="D17" s="42">
         <f t="shared" si="7"/>
         <v>46120</v>
@@ -3342,7 +3344,9 @@
       <c r="B18" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="C18" s="15"/>
+      <c r="C18" s="15">
+        <v>1</v>
+      </c>
       <c r="D18" s="42">
         <f t="shared" si="7"/>
         <v>46121</v>
@@ -3418,7 +3422,9 @@
       <c r="B19" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="C19" s="15"/>
+      <c r="C19" s="15">
+        <v>1</v>
+      </c>
       <c r="D19" s="42">
         <f t="shared" si="7"/>
         <v>46124</v>
@@ -3491,7 +3497,9 @@
       <c r="B20" s="31" t="s">
         <v>34</v>
       </c>
-      <c r="C20" s="15"/>
+      <c r="C20" s="15">
+        <v>1</v>
+      </c>
       <c r="D20" s="42">
         <f t="shared" si="7"/>
         <v>46127</v>
@@ -3564,7 +3572,9 @@
       <c r="B21" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="C21" s="15"/>
+      <c r="C21" s="15">
+        <v>1</v>
+      </c>
       <c r="D21" s="42">
         <f t="shared" si="7"/>
         <v>46129</v>
@@ -3637,7 +3647,9 @@
       <c r="B22" s="31" t="s">
         <v>36</v>
       </c>
-      <c r="C22" s="15"/>
+      <c r="C22" s="15">
+        <v>1</v>
+      </c>
       <c r="D22" s="42">
         <f t="shared" si="7"/>
         <v>46131</v>
@@ -3710,7 +3722,9 @@
       <c r="B23" s="31" t="s">
         <v>37</v>
       </c>
-      <c r="C23" s="15"/>
+      <c r="C23" s="15">
+        <v>0</v>
+      </c>
       <c r="D23" s="42">
         <f t="shared" si="7"/>
         <v>46132</v>
@@ -6438,35 +6452,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Image>
-    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
-    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </ImageTagsTaxHTField>
-    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
-    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="24" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2d714a3296df14eba7a100bb665443ca">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="49549bf45bfbbfb6cffed527380e77e1" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -6754,34 +6739,36 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5144944C-1F1D-4162-962A-96F3FC8455D8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="16c05727-aa75-4e4a-9b5f-8a80a1165891"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8FE8ED85-58B3-4608-8E91-0433556D50CE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Image>
+    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
+    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </ImageTagsTaxHTField>
+    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
+    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{708DBB9E-6D89-4A94-9DC5-964B7833E11C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6800,4 +6787,31 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8FE8ED85-58B3-4608-8E91-0433556D50CE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5144944C-1F1D-4162-962A-96F3FC8455D8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="16c05727-aa75-4e4a-9b5f-8a80a1165891"/>
+    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Modificacion en fechas de diagrama de GANTT
</commit_message>
<xml_diff>
--- a/diagramaGANTT.xlsx
+++ b/diagramaGANTT.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12AC9A70-4E22-4DB7-AC1D-119728C8EC2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{169D5D92-334B-4D19-9601-95BF28CF6789}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="53">
   <si>
     <t>Cree una programación para un proyecto en esta hoja de cálculo.
 Escriba el título de este proyecto en la celda B1. 
@@ -208,46 +208,10 @@
     <t>Probar que todo funciona</t>
   </si>
   <si>
-    <t>Probar registro de usuario</t>
-  </si>
-  <si>
-    <t>Probar inicio de sesión</t>
-  </si>
-  <si>
-    <t>Probar edición de perfil</t>
-  </si>
-  <si>
-    <t>Probar cierre de sesión</t>
-  </si>
-  <si>
-    <t>Probar catálogo y búsqueda</t>
-  </si>
-  <si>
-    <t>Probar filtros</t>
-  </si>
-  <si>
-    <t>Probar detalle de producto</t>
-  </si>
-  <si>
-    <t>Probar favoritos</t>
-  </si>
-  <si>
-    <t>Probar cookies (productos visitados)</t>
-  </si>
-  <si>
-    <t>Probar cambio de idioma</t>
-  </si>
-  <si>
     <t>DESPLIEGUE</t>
   </si>
   <si>
-    <t>Comprar dominio y hosting</t>
-  </si>
-  <si>
     <t>Subir el código</t>
-  </si>
-  <si>
-    <t>Configurar base de datos</t>
   </si>
   <si>
     <t>Probar que la web online funciona</t>
@@ -263,6 +227,12 @@
   </si>
   <si>
     <t>Entrega final</t>
+  </si>
+  <si>
+    <t>Panel de administración de zapatillas - RFP-016</t>
+  </si>
+  <si>
+    <t>Comprar dominio</t>
   </si>
 </sst>
 </file>
@@ -1885,7 +1855,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BK50"/>
+  <dimension ref="A1:BK40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.7109375" style="25" customWidth="1"/>
@@ -2580,7 +2550,7 @@
       <c r="E8" s="38"/>
       <c r="F8" s="9"/>
       <c r="G8" s="9" t="str">
-        <f t="shared" ref="G8:G50" si="6">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+        <f t="shared" ref="G8:G40" si="6">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v/>
       </c>
       <c r="H8" s="22"/>
@@ -3036,7 +3006,7 @@
         <v>1</v>
       </c>
       <c r="D14" s="42">
-        <f t="shared" ref="D14:D28" si="7">E13+1</f>
+        <f t="shared" ref="D14:D29" si="7">E13+1</f>
         <v>46117</v>
       </c>
       <c r="E14" s="42">
@@ -3342,13 +3312,13 @@
     <row r="18" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="25"/>
       <c r="B18" s="31" t="s">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="C18" s="15">
         <v>1</v>
       </c>
       <c r="D18" s="42">
-        <f t="shared" si="7"/>
+        <f>E17+1</f>
         <v>46121</v>
       </c>
       <c r="E18" s="42">
@@ -3356,10 +3326,7 @@
         <v>46123</v>
       </c>
       <c r="F18" s="9"/>
-      <c r="G18" s="9">
-        <f t="shared" si="6"/>
-        <v>3</v>
-      </c>
+      <c r="G18" s="9"/>
       <c r="H18" s="22"/>
       <c r="I18" s="22"/>
       <c r="J18" s="22"/>
@@ -3420,21 +3387,24 @@
     <row r="19" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="25"/>
       <c r="B19" s="31" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C19" s="15">
         <v>1</v>
       </c>
       <c r="D19" s="42">
-        <f t="shared" si="7"/>
-        <v>46124</v>
+        <f>E17+1</f>
+        <v>46121</v>
       </c>
       <c r="E19" s="42">
         <f>D19+2</f>
-        <v>46126</v>
+        <v>46123</v>
       </c>
       <c r="F19" s="9"/>
-      <c r="G19" s="9"/>
+      <c r="G19" s="9">
+        <f t="shared" si="6"/>
+        <v>3</v>
+      </c>
       <c r="H19" s="22"/>
       <c r="I19" s="22"/>
       <c r="J19" s="22"/>
@@ -3495,18 +3465,18 @@
     <row r="20" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="25"/>
       <c r="B20" s="31" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C20" s="15">
         <v>1</v>
       </c>
       <c r="D20" s="42">
         <f t="shared" si="7"/>
-        <v>46127</v>
+        <v>46124</v>
       </c>
       <c r="E20" s="42">
-        <f>D20+1</f>
-        <v>46128</v>
+        <f>D20+2</f>
+        <v>46126</v>
       </c>
       <c r="F20" s="9"/>
       <c r="G20" s="9"/>
@@ -3570,18 +3540,18 @@
     <row r="21" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="25"/>
       <c r="B21" s="31" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C21" s="15">
         <v>1</v>
       </c>
       <c r="D21" s="42">
         <f t="shared" si="7"/>
-        <v>46129</v>
+        <v>46127</v>
       </c>
       <c r="E21" s="42">
         <f>D21+1</f>
-        <v>46130</v>
+        <v>46128</v>
       </c>
       <c r="F21" s="9"/>
       <c r="G21" s="9"/>
@@ -3645,18 +3615,18 @@
     <row r="22" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="25"/>
       <c r="B22" s="31" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C22" s="15">
         <v>1</v>
       </c>
       <c r="D22" s="42">
         <f t="shared" si="7"/>
-        <v>46131</v>
+        <v>46129</v>
       </c>
       <c r="E22" s="42">
-        <f>D22</f>
-        <v>46131</v>
+        <f>D22+1</f>
+        <v>46130</v>
       </c>
       <c r="F22" s="9"/>
       <c r="G22" s="9"/>
@@ -3720,18 +3690,18 @@
     <row r="23" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="25"/>
       <c r="B23" s="31" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C23" s="15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D23" s="42">
         <f t="shared" si="7"/>
-        <v>46132</v>
+        <v>46131</v>
       </c>
       <c r="E23" s="42">
-        <f>D23+2</f>
-        <v>46134</v>
+        <f>D23</f>
+        <v>46131</v>
       </c>
       <c r="F23" s="9"/>
       <c r="G23" s="9"/>
@@ -3795,16 +3765,18 @@
     <row r="24" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="25"/>
       <c r="B24" s="31" t="s">
-        <v>38</v>
-      </c>
-      <c r="C24" s="15"/>
+        <v>37</v>
+      </c>
+      <c r="C24" s="15">
+        <v>1</v>
+      </c>
       <c r="D24" s="42">
         <f t="shared" si="7"/>
-        <v>46135</v>
+        <v>46132</v>
       </c>
       <c r="E24" s="42">
         <f>D24+1</f>
-        <v>46136</v>
+        <v>46133</v>
       </c>
       <c r="F24" s="9"/>
       <c r="G24" s="9"/>
@@ -3868,16 +3840,18 @@
     <row r="25" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="25"/>
       <c r="B25" s="31" t="s">
-        <v>39</v>
-      </c>
-      <c r="C25" s="15"/>
+        <v>38</v>
+      </c>
+      <c r="C25" s="15">
+        <v>1</v>
+      </c>
       <c r="D25" s="42">
-        <f t="shared" si="7"/>
-        <v>46137</v>
+        <f>E23+1</f>
+        <v>46132</v>
       </c>
       <c r="E25" s="42">
         <f>D25+1</f>
-        <v>46138</v>
+        <v>46133</v>
       </c>
       <c r="F25" s="9"/>
       <c r="G25" s="9"/>
@@ -3941,16 +3915,16 @@
     <row r="26" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="25"/>
       <c r="B26" s="31" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C26" s="15"/>
       <c r="D26" s="42">
         <f t="shared" si="7"/>
-        <v>46139</v>
+        <v>46134</v>
       </c>
       <c r="E26" s="42">
         <f>D26+1</f>
-        <v>46140</v>
+        <v>46135</v>
       </c>
       <c r="F26" s="9"/>
       <c r="G26" s="9"/>
@@ -4014,16 +3988,16 @@
     <row r="27" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="25"/>
       <c r="B27" s="31" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C27" s="15"/>
       <c r="D27" s="42">
         <f t="shared" si="7"/>
-        <v>46141</v>
+        <v>46136</v>
       </c>
       <c r="E27" s="42">
-        <f>D27+2</f>
-        <v>46143</v>
+        <f>D27+1</f>
+        <v>46137</v>
       </c>
       <c r="F27" s="9"/>
       <c r="G27" s="9"/>
@@ -4087,16 +4061,16 @@
     <row r="28" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="25"/>
       <c r="B28" s="31" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C28" s="15"/>
       <c r="D28" s="42">
         <f t="shared" si="7"/>
-        <v>46144</v>
+        <v>46138</v>
       </c>
       <c r="E28" s="42">
-        <f>D28+2</f>
-        <v>46146</v>
+        <f>D28+1</f>
+        <v>46139</v>
       </c>
       <c r="F28" s="9"/>
       <c r="G28" s="9"/>
@@ -4158,20 +4132,21 @@
       <c r="BK28" s="22"/>
     </row>
     <row r="29" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="25" t="s">
-        <v>18</v>
-      </c>
-      <c r="B29" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="C29" s="17"/>
-      <c r="D29" s="43"/>
-      <c r="E29" s="44"/>
+      <c r="A29" s="25"/>
+      <c r="B29" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="C29" s="15"/>
+      <c r="D29" s="42">
+        <f t="shared" si="7"/>
+        <v>46140</v>
+      </c>
+      <c r="E29" s="42">
+        <f>D29</f>
+        <v>46140</v>
+      </c>
       <c r="F29" s="9"/>
-      <c r="G29" s="9" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
+      <c r="G29" s="9"/>
       <c r="H29" s="22"/>
       <c r="I29" s="22"/>
       <c r="J29" s="22"/>
@@ -4230,23 +4205,19 @@
       <c r="BK29" s="22"/>
     </row>
     <row r="30" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="25"/>
-      <c r="B30" s="32" t="s">
-        <v>43</v>
-      </c>
-      <c r="C30" s="18"/>
-      <c r="D30" s="45">
-        <f>E28+1</f>
-        <v>46147</v>
-      </c>
-      <c r="E30" s="45">
-        <f t="shared" ref="E30:E40" si="8">D30+1</f>
-        <v>46148</v>
-      </c>
+      <c r="A30" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="B30" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="C30" s="17"/>
+      <c r="D30" s="43"/>
+      <c r="E30" s="44"/>
       <c r="F30" s="9"/>
-      <c r="G30" s="9">
+      <c r="G30" s="9" t="str">
         <f t="shared" si="6"/>
-        <v>2</v>
+        <v/>
       </c>
       <c r="H30" s="22"/>
       <c r="I30" s="22"/>
@@ -4308,21 +4279,21 @@
     <row r="31" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="25"/>
       <c r="B31" s="32" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C31" s="18"/>
       <c r="D31" s="45">
-        <f>D30</f>
-        <v>46147</v>
+        <f>E29+1</f>
+        <v>46141</v>
       </c>
       <c r="E31" s="45">
-        <f t="shared" si="8"/>
-        <v>46148</v>
+        <f>D31</f>
+        <v>46141</v>
       </c>
       <c r="F31" s="9"/>
       <c r="G31" s="9">
         <f t="shared" si="6"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H31" s="22"/>
       <c r="I31" s="22"/>
@@ -4382,23 +4353,19 @@
       <c r="BK31" s="22"/>
     </row>
     <row r="32" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="25"/>
-      <c r="B32" s="32" t="s">
-        <v>45</v>
-      </c>
-      <c r="C32" s="18"/>
-      <c r="D32" s="45">
-        <f>D31</f>
-        <v>46147</v>
-      </c>
-      <c r="E32" s="45">
-        <f t="shared" si="8"/>
-        <v>46148</v>
-      </c>
+      <c r="A32" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="B32" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="C32" s="20"/>
+      <c r="D32" s="46"/>
+      <c r="E32" s="47"/>
       <c r="F32" s="9"/>
-      <c r="G32" s="9">
+      <c r="G32" s="9" t="str">
         <f t="shared" si="6"/>
-        <v>2</v>
+        <v/>
       </c>
       <c r="H32" s="22"/>
       <c r="I32" s="22"/>
@@ -4459,22 +4426,22 @@
     </row>
     <row r="33" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="25"/>
-      <c r="B33" s="32" t="s">
-        <v>46</v>
-      </c>
-      <c r="C33" s="18"/>
-      <c r="D33" s="45">
-        <f>D32</f>
-        <v>46147</v>
-      </c>
-      <c r="E33" s="45">
-        <f t="shared" si="8"/>
-        <v>46148</v>
+      <c r="B33" s="33" t="s">
+        <v>52</v>
+      </c>
+      <c r="C33" s="21"/>
+      <c r="D33" s="48">
+        <f>E31+1</f>
+        <v>46142</v>
+      </c>
+      <c r="E33" s="48">
+        <f>D33</f>
+        <v>46142</v>
       </c>
       <c r="F33" s="9"/>
       <c r="G33" s="9">
         <f t="shared" si="6"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H33" s="22"/>
       <c r="I33" s="22"/>
@@ -4535,22 +4502,22 @@
     </row>
     <row r="34" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="25"/>
-      <c r="B34" s="32" t="s">
-        <v>47</v>
-      </c>
-      <c r="C34" s="18"/>
-      <c r="D34" s="45">
-        <f>D33</f>
-        <v>46147</v>
-      </c>
-      <c r="E34" s="45">
-        <f t="shared" si="8"/>
-        <v>46148</v>
+      <c r="B34" s="33" t="s">
+        <v>45</v>
+      </c>
+      <c r="C34" s="21"/>
+      <c r="D34" s="48">
+        <f>E33+1</f>
+        <v>46143</v>
+      </c>
+      <c r="E34" s="48">
+        <f>D34+2</f>
+        <v>46145</v>
       </c>
       <c r="F34" s="9"/>
       <c r="G34" s="9">
         <f t="shared" si="6"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H34" s="22"/>
       <c r="I34" s="22"/>
@@ -4611,20 +4578,23 @@
     </row>
     <row r="35" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="25"/>
-      <c r="B35" s="32" t="s">
-        <v>48</v>
-      </c>
-      <c r="C35" s="18"/>
-      <c r="D35" s="45">
+      <c r="B35" s="33" t="s">
+        <v>46</v>
+      </c>
+      <c r="C35" s="21"/>
+      <c r="D35" s="48">
         <f>E34+1</f>
-        <v>46149</v>
-      </c>
-      <c r="E35" s="45">
-        <f t="shared" si="8"/>
-        <v>46150</v>
+        <v>46146</v>
+      </c>
+      <c r="E35" s="48">
+        <f>D35</f>
+        <v>46146</v>
       </c>
       <c r="F35" s="9"/>
-      <c r="G35" s="9"/>
+      <c r="G35" s="9">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
       <c r="H35" s="22"/>
       <c r="I35" s="22"/>
       <c r="J35" s="22"/>
@@ -4684,18 +4654,12 @@
     </row>
     <row r="36" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="25"/>
-      <c r="B36" s="32" t="s">
-        <v>49</v>
-      </c>
-      <c r="C36" s="18"/>
-      <c r="D36" s="45">
-        <f>D35</f>
-        <v>46149</v>
-      </c>
-      <c r="E36" s="45">
-        <f t="shared" si="8"/>
-        <v>46150</v>
-      </c>
+      <c r="B36" s="57" t="s">
+        <v>22</v>
+      </c>
+      <c r="C36" s="58"/>
+      <c r="D36" s="59"/>
+      <c r="E36" s="60"/>
       <c r="F36" s="9"/>
       <c r="G36" s="9"/>
       <c r="H36" s="22"/>
@@ -4757,17 +4721,17 @@
     </row>
     <row r="37" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="25"/>
-      <c r="B37" s="32" t="s">
-        <v>50</v>
-      </c>
-      <c r="C37" s="18"/>
-      <c r="D37" s="45">
-        <f>D36</f>
-        <v>46149</v>
-      </c>
-      <c r="E37" s="45">
-        <f t="shared" si="8"/>
-        <v>46150</v>
+      <c r="B37" s="62" t="s">
+        <v>47</v>
+      </c>
+      <c r="C37" s="61"/>
+      <c r="D37" s="63">
+        <f>E35+1</f>
+        <v>46147</v>
+      </c>
+      <c r="E37" s="63">
+        <f>D37+1</f>
+        <v>46148</v>
       </c>
       <c r="F37" s="9"/>
       <c r="G37" s="9"/>
@@ -4830,16 +4794,16 @@
     </row>
     <row r="38" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="25"/>
-      <c r="B38" s="32" t="s">
-        <v>51</v>
-      </c>
-      <c r="C38" s="18"/>
-      <c r="D38" s="45">
-        <f>D37</f>
+      <c r="B38" s="62" t="s">
+        <v>48</v>
+      </c>
+      <c r="C38" s="61"/>
+      <c r="D38" s="63">
+        <f>E37+1</f>
         <v>46149</v>
       </c>
-      <c r="E38" s="45">
-        <f t="shared" si="8"/>
+      <c r="E38" s="63">
+        <f>D38+1</f>
         <v>46150</v>
       </c>
       <c r="F38" s="9"/>
@@ -4903,17 +4867,17 @@
     </row>
     <row r="39" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="25"/>
-      <c r="B39" s="32" t="s">
-        <v>52</v>
-      </c>
-      <c r="C39" s="18"/>
-      <c r="D39" s="45">
-        <f>D38</f>
-        <v>46149</v>
-      </c>
-      <c r="E39" s="45">
-        <f t="shared" si="8"/>
-        <v>46150</v>
+      <c r="B39" s="62" t="s">
+        <v>49</v>
+      </c>
+      <c r="C39" s="61"/>
+      <c r="D39" s="63">
+        <f>E38+1</f>
+        <v>46151</v>
+      </c>
+      <c r="E39" s="63">
+        <f>D39+1</f>
+        <v>46152</v>
       </c>
       <c r="F39" s="9"/>
       <c r="G39" s="9"/>
@@ -4975,21 +4939,26 @@
       <c r="BK39" s="22"/>
     </row>
     <row r="40" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="25"/>
-      <c r="B40" s="32" t="s">
-        <v>53</v>
-      </c>
-      <c r="C40" s="18"/>
-      <c r="D40" s="45">
+      <c r="A40" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="B40" s="62" t="s">
+        <v>50</v>
+      </c>
+      <c r="C40" s="61"/>
+      <c r="D40" s="63">
         <f>E39+1</f>
-        <v>46151</v>
-      </c>
-      <c r="E40" s="45">
-        <f t="shared" si="8"/>
-        <v>46152</v>
+        <v>46153</v>
+      </c>
+      <c r="E40" s="63">
+        <f>D40+3</f>
+        <v>46156</v>
       </c>
       <c r="F40" s="9"/>
-      <c r="G40" s="9"/>
+      <c r="G40" s="9">
+        <f t="shared" si="6"/>
+        <v>4</v>
+      </c>
       <c r="H40" s="22"/>
       <c r="I40" s="22"/>
       <c r="J40" s="22"/>
@@ -5047,746 +5016,6 @@
       <c r="BJ40" s="22"/>
       <c r="BK40" s="22"/>
     </row>
-    <row r="41" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="25" t="s">
-        <v>18</v>
-      </c>
-      <c r="B41" s="19" t="s">
-        <v>54</v>
-      </c>
-      <c r="C41" s="20"/>
-      <c r="D41" s="46"/>
-      <c r="E41" s="47"/>
-      <c r="F41" s="9"/>
-      <c r="G41" s="9" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="H41" s="22"/>
-      <c r="I41" s="22"/>
-      <c r="J41" s="22"/>
-      <c r="K41" s="22"/>
-      <c r="L41" s="22"/>
-      <c r="M41" s="22"/>
-      <c r="N41" s="22"/>
-      <c r="O41" s="22"/>
-      <c r="P41" s="22"/>
-      <c r="Q41" s="22"/>
-      <c r="R41" s="22"/>
-      <c r="S41" s="22"/>
-      <c r="T41" s="22"/>
-      <c r="U41" s="22"/>
-      <c r="V41" s="22"/>
-      <c r="W41" s="22"/>
-      <c r="X41" s="22"/>
-      <c r="Y41" s="22"/>
-      <c r="Z41" s="22"/>
-      <c r="AA41" s="22"/>
-      <c r="AB41" s="22"/>
-      <c r="AC41" s="22"/>
-      <c r="AD41" s="22"/>
-      <c r="AE41" s="22"/>
-      <c r="AF41" s="22"/>
-      <c r="AG41" s="22"/>
-      <c r="AH41" s="22"/>
-      <c r="AI41" s="22"/>
-      <c r="AJ41" s="22"/>
-      <c r="AK41" s="22"/>
-      <c r="AL41" s="22"/>
-      <c r="AM41" s="22"/>
-      <c r="AN41" s="22"/>
-      <c r="AO41" s="22"/>
-      <c r="AP41" s="22"/>
-      <c r="AQ41" s="22"/>
-      <c r="AR41" s="22"/>
-      <c r="AS41" s="22"/>
-      <c r="AT41" s="22"/>
-      <c r="AU41" s="22"/>
-      <c r="AV41" s="22"/>
-      <c r="AW41" s="22"/>
-      <c r="AX41" s="22"/>
-      <c r="AY41" s="22"/>
-      <c r="AZ41" s="22"/>
-      <c r="BA41" s="22"/>
-      <c r="BB41" s="22"/>
-      <c r="BC41" s="22"/>
-      <c r="BD41" s="22"/>
-      <c r="BE41" s="22"/>
-      <c r="BF41" s="22"/>
-      <c r="BG41" s="22"/>
-      <c r="BH41" s="22"/>
-      <c r="BI41" s="22"/>
-      <c r="BJ41" s="22"/>
-      <c r="BK41" s="22"/>
-    </row>
-    <row r="42" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="25"/>
-      <c r="B42" s="33" t="s">
-        <v>55</v>
-      </c>
-      <c r="C42" s="21"/>
-      <c r="D42" s="48">
-        <f>E40+1</f>
-        <v>46153</v>
-      </c>
-      <c r="E42" s="48">
-        <f>D42</f>
-        <v>46153</v>
-      </c>
-      <c r="F42" s="9"/>
-      <c r="G42" s="9">
-        <f t="shared" si="6"/>
-        <v>1</v>
-      </c>
-      <c r="H42" s="22"/>
-      <c r="I42" s="22"/>
-      <c r="J42" s="22"/>
-      <c r="K42" s="22"/>
-      <c r="L42" s="22"/>
-      <c r="M42" s="22"/>
-      <c r="N42" s="22"/>
-      <c r="O42" s="22"/>
-      <c r="P42" s="22"/>
-      <c r="Q42" s="22"/>
-      <c r="R42" s="22"/>
-      <c r="S42" s="22"/>
-      <c r="T42" s="22"/>
-      <c r="U42" s="22"/>
-      <c r="V42" s="22"/>
-      <c r="W42" s="22"/>
-      <c r="X42" s="22"/>
-      <c r="Y42" s="22"/>
-      <c r="Z42" s="22"/>
-      <c r="AA42" s="22"/>
-      <c r="AB42" s="22"/>
-      <c r="AC42" s="22"/>
-      <c r="AD42" s="22"/>
-      <c r="AE42" s="22"/>
-      <c r="AF42" s="22"/>
-      <c r="AG42" s="22"/>
-      <c r="AH42" s="22"/>
-      <c r="AI42" s="22"/>
-      <c r="AJ42" s="22"/>
-      <c r="AK42" s="22"/>
-      <c r="AL42" s="22"/>
-      <c r="AM42" s="22"/>
-      <c r="AN42" s="22"/>
-      <c r="AO42" s="22"/>
-      <c r="AP42" s="22"/>
-      <c r="AQ42" s="22"/>
-      <c r="AR42" s="22"/>
-      <c r="AS42" s="22"/>
-      <c r="AT42" s="22"/>
-      <c r="AU42" s="22"/>
-      <c r="AV42" s="22"/>
-      <c r="AW42" s="22"/>
-      <c r="AX42" s="22"/>
-      <c r="AY42" s="22"/>
-      <c r="AZ42" s="22"/>
-      <c r="BA42" s="22"/>
-      <c r="BB42" s="22"/>
-      <c r="BC42" s="22"/>
-      <c r="BD42" s="22"/>
-      <c r="BE42" s="22"/>
-      <c r="BF42" s="22"/>
-      <c r="BG42" s="22"/>
-      <c r="BH42" s="22"/>
-      <c r="BI42" s="22"/>
-      <c r="BJ42" s="22"/>
-      <c r="BK42" s="22"/>
-    </row>
-    <row r="43" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="25"/>
-      <c r="B43" s="33" t="s">
-        <v>56</v>
-      </c>
-      <c r="C43" s="21"/>
-      <c r="D43" s="48">
-        <f>E42+1</f>
-        <v>46154</v>
-      </c>
-      <c r="E43" s="48">
-        <f>D43+1</f>
-        <v>46155</v>
-      </c>
-      <c r="F43" s="9"/>
-      <c r="G43" s="9">
-        <f t="shared" si="6"/>
-        <v>2</v>
-      </c>
-      <c r="H43" s="22"/>
-      <c r="I43" s="22"/>
-      <c r="J43" s="22"/>
-      <c r="K43" s="22"/>
-      <c r="L43" s="22"/>
-      <c r="M43" s="22"/>
-      <c r="N43" s="22"/>
-      <c r="O43" s="22"/>
-      <c r="P43" s="22"/>
-      <c r="Q43" s="22"/>
-      <c r="R43" s="22"/>
-      <c r="S43" s="22"/>
-      <c r="T43" s="22"/>
-      <c r="U43" s="22"/>
-      <c r="V43" s="22"/>
-      <c r="W43" s="22"/>
-      <c r="X43" s="22"/>
-      <c r="Y43" s="22"/>
-      <c r="Z43" s="22"/>
-      <c r="AA43" s="22"/>
-      <c r="AB43" s="22"/>
-      <c r="AC43" s="22"/>
-      <c r="AD43" s="22"/>
-      <c r="AE43" s="22"/>
-      <c r="AF43" s="22"/>
-      <c r="AG43" s="22"/>
-      <c r="AH43" s="22"/>
-      <c r="AI43" s="22"/>
-      <c r="AJ43" s="22"/>
-      <c r="AK43" s="22"/>
-      <c r="AL43" s="22"/>
-      <c r="AM43" s="22"/>
-      <c r="AN43" s="22"/>
-      <c r="AO43" s="22"/>
-      <c r="AP43" s="22"/>
-      <c r="AQ43" s="22"/>
-      <c r="AR43" s="22"/>
-      <c r="AS43" s="22"/>
-      <c r="AT43" s="22"/>
-      <c r="AU43" s="22"/>
-      <c r="AV43" s="22"/>
-      <c r="AW43" s="22"/>
-      <c r="AX43" s="22"/>
-      <c r="AY43" s="22"/>
-      <c r="AZ43" s="22"/>
-      <c r="BA43" s="22"/>
-      <c r="BB43" s="22"/>
-      <c r="BC43" s="22"/>
-      <c r="BD43" s="22"/>
-      <c r="BE43" s="22"/>
-      <c r="BF43" s="22"/>
-      <c r="BG43" s="22"/>
-      <c r="BH43" s="22"/>
-      <c r="BI43" s="22"/>
-      <c r="BJ43" s="22"/>
-      <c r="BK43" s="22"/>
-    </row>
-    <row r="44" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="25"/>
-      <c r="B44" s="33" t="s">
-        <v>57</v>
-      </c>
-      <c r="C44" s="21"/>
-      <c r="D44" s="48">
-        <f>E43+1</f>
-        <v>46156</v>
-      </c>
-      <c r="E44" s="48">
-        <f>D44+1</f>
-        <v>46157</v>
-      </c>
-      <c r="F44" s="9"/>
-      <c r="G44" s="9">
-        <f t="shared" si="6"/>
-        <v>2</v>
-      </c>
-      <c r="H44" s="22"/>
-      <c r="I44" s="22"/>
-      <c r="J44" s="22"/>
-      <c r="K44" s="22"/>
-      <c r="L44" s="22"/>
-      <c r="M44" s="22"/>
-      <c r="N44" s="22"/>
-      <c r="O44" s="22"/>
-      <c r="P44" s="22"/>
-      <c r="Q44" s="22"/>
-      <c r="R44" s="22"/>
-      <c r="S44" s="22"/>
-      <c r="T44" s="22"/>
-      <c r="U44" s="22"/>
-      <c r="V44" s="22"/>
-      <c r="W44" s="22"/>
-      <c r="X44" s="22"/>
-      <c r="Y44" s="22"/>
-      <c r="Z44" s="22"/>
-      <c r="AA44" s="22"/>
-      <c r="AB44" s="22"/>
-      <c r="AC44" s="22"/>
-      <c r="AD44" s="22"/>
-      <c r="AE44" s="22"/>
-      <c r="AF44" s="22"/>
-      <c r="AG44" s="22"/>
-      <c r="AH44" s="22"/>
-      <c r="AI44" s="22"/>
-      <c r="AJ44" s="22"/>
-      <c r="AK44" s="22"/>
-      <c r="AL44" s="22"/>
-      <c r="AM44" s="22"/>
-      <c r="AN44" s="22"/>
-      <c r="AO44" s="22"/>
-      <c r="AP44" s="22"/>
-      <c r="AQ44" s="22"/>
-      <c r="AR44" s="22"/>
-      <c r="AS44" s="22"/>
-      <c r="AT44" s="22"/>
-      <c r="AU44" s="22"/>
-      <c r="AV44" s="22"/>
-      <c r="AW44" s="22"/>
-      <c r="AX44" s="22"/>
-      <c r="AY44" s="22"/>
-      <c r="AZ44" s="22"/>
-      <c r="BA44" s="22"/>
-      <c r="BB44" s="22"/>
-      <c r="BC44" s="22"/>
-      <c r="BD44" s="22"/>
-      <c r="BE44" s="22"/>
-      <c r="BF44" s="22"/>
-      <c r="BG44" s="22"/>
-      <c r="BH44" s="22"/>
-      <c r="BI44" s="22"/>
-      <c r="BJ44" s="22"/>
-      <c r="BK44" s="22"/>
-    </row>
-    <row r="45" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="25"/>
-      <c r="B45" s="33" t="s">
-        <v>58</v>
-      </c>
-      <c r="C45" s="21"/>
-      <c r="D45" s="48">
-        <f>E44+1</f>
-        <v>46158</v>
-      </c>
-      <c r="E45" s="48">
-        <f>D45+1</f>
-        <v>46159</v>
-      </c>
-      <c r="F45" s="9"/>
-      <c r="G45" s="9">
-        <f t="shared" si="6"/>
-        <v>2</v>
-      </c>
-      <c r="H45" s="22"/>
-      <c r="I45" s="22"/>
-      <c r="J45" s="22"/>
-      <c r="K45" s="22"/>
-      <c r="L45" s="22"/>
-      <c r="M45" s="22"/>
-      <c r="N45" s="22"/>
-      <c r="O45" s="22"/>
-      <c r="P45" s="22"/>
-      <c r="Q45" s="22"/>
-      <c r="R45" s="22"/>
-      <c r="S45" s="22"/>
-      <c r="T45" s="22"/>
-      <c r="U45" s="22"/>
-      <c r="V45" s="22"/>
-      <c r="W45" s="22"/>
-      <c r="X45" s="22"/>
-      <c r="Y45" s="22"/>
-      <c r="Z45" s="22"/>
-      <c r="AA45" s="22"/>
-      <c r="AB45" s="22"/>
-      <c r="AC45" s="22"/>
-      <c r="AD45" s="22"/>
-      <c r="AE45" s="22"/>
-      <c r="AF45" s="22"/>
-      <c r="AG45" s="22"/>
-      <c r="AH45" s="22"/>
-      <c r="AI45" s="22"/>
-      <c r="AJ45" s="22"/>
-      <c r="AK45" s="22"/>
-      <c r="AL45" s="22"/>
-      <c r="AM45" s="22"/>
-      <c r="AN45" s="22"/>
-      <c r="AO45" s="22"/>
-      <c r="AP45" s="22"/>
-      <c r="AQ45" s="22"/>
-      <c r="AR45" s="22"/>
-      <c r="AS45" s="22"/>
-      <c r="AT45" s="22"/>
-      <c r="AU45" s="22"/>
-      <c r="AV45" s="22"/>
-      <c r="AW45" s="22"/>
-      <c r="AX45" s="22"/>
-      <c r="AY45" s="22"/>
-      <c r="AZ45" s="22"/>
-      <c r="BA45" s="22"/>
-      <c r="BB45" s="22"/>
-      <c r="BC45" s="22"/>
-      <c r="BD45" s="22"/>
-      <c r="BE45" s="22"/>
-      <c r="BF45" s="22"/>
-      <c r="BG45" s="22"/>
-      <c r="BH45" s="22"/>
-      <c r="BI45" s="22"/>
-      <c r="BJ45" s="22"/>
-      <c r="BK45" s="22"/>
-    </row>
-    <row r="46" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="25"/>
-      <c r="B46" s="57" t="s">
-        <v>22</v>
-      </c>
-      <c r="C46" s="58"/>
-      <c r="D46" s="59"/>
-      <c r="E46" s="60"/>
-      <c r="F46" s="9"/>
-      <c r="G46" s="9"/>
-      <c r="H46" s="22"/>
-      <c r="I46" s="22"/>
-      <c r="J46" s="22"/>
-      <c r="K46" s="22"/>
-      <c r="L46" s="22"/>
-      <c r="M46" s="22"/>
-      <c r="N46" s="22"/>
-      <c r="O46" s="22"/>
-      <c r="P46" s="22"/>
-      <c r="Q46" s="22"/>
-      <c r="R46" s="22"/>
-      <c r="S46" s="22"/>
-      <c r="T46" s="22"/>
-      <c r="U46" s="22"/>
-      <c r="V46" s="22"/>
-      <c r="W46" s="22"/>
-      <c r="X46" s="22"/>
-      <c r="Y46" s="22"/>
-      <c r="Z46" s="22"/>
-      <c r="AA46" s="22"/>
-      <c r="AB46" s="22"/>
-      <c r="AC46" s="22"/>
-      <c r="AD46" s="22"/>
-      <c r="AE46" s="22"/>
-      <c r="AF46" s="22"/>
-      <c r="AG46" s="22"/>
-      <c r="AH46" s="22"/>
-      <c r="AI46" s="22"/>
-      <c r="AJ46" s="22"/>
-      <c r="AK46" s="22"/>
-      <c r="AL46" s="22"/>
-      <c r="AM46" s="22"/>
-      <c r="AN46" s="22"/>
-      <c r="AO46" s="22"/>
-      <c r="AP46" s="22"/>
-      <c r="AQ46" s="22"/>
-      <c r="AR46" s="22"/>
-      <c r="AS46" s="22"/>
-      <c r="AT46" s="22"/>
-      <c r="AU46" s="22"/>
-      <c r="AV46" s="22"/>
-      <c r="AW46" s="22"/>
-      <c r="AX46" s="22"/>
-      <c r="AY46" s="22"/>
-      <c r="AZ46" s="22"/>
-      <c r="BA46" s="22"/>
-      <c r="BB46" s="22"/>
-      <c r="BC46" s="22"/>
-      <c r="BD46" s="22"/>
-      <c r="BE46" s="22"/>
-      <c r="BF46" s="22"/>
-      <c r="BG46" s="22"/>
-      <c r="BH46" s="22"/>
-      <c r="BI46" s="22"/>
-      <c r="BJ46" s="22"/>
-      <c r="BK46" s="22"/>
-    </row>
-    <row r="47" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="25"/>
-      <c r="B47" s="62" t="s">
-        <v>59</v>
-      </c>
-      <c r="C47" s="61"/>
-      <c r="D47" s="63">
-        <f>E45+1</f>
-        <v>46160</v>
-      </c>
-      <c r="E47" s="63">
-        <f>D47+1</f>
-        <v>46161</v>
-      </c>
-      <c r="F47" s="9"/>
-      <c r="G47" s="9"/>
-      <c r="H47" s="22"/>
-      <c r="I47" s="22"/>
-      <c r="J47" s="22"/>
-      <c r="K47" s="22"/>
-      <c r="L47" s="22"/>
-      <c r="M47" s="22"/>
-      <c r="N47" s="22"/>
-      <c r="O47" s="22"/>
-      <c r="P47" s="22"/>
-      <c r="Q47" s="22"/>
-      <c r="R47" s="22"/>
-      <c r="S47" s="22"/>
-      <c r="T47" s="22"/>
-      <c r="U47" s="22"/>
-      <c r="V47" s="22"/>
-      <c r="W47" s="22"/>
-      <c r="X47" s="22"/>
-      <c r="Y47" s="22"/>
-      <c r="Z47" s="22"/>
-      <c r="AA47" s="22"/>
-      <c r="AB47" s="22"/>
-      <c r="AC47" s="22"/>
-      <c r="AD47" s="22"/>
-      <c r="AE47" s="22"/>
-      <c r="AF47" s="22"/>
-      <c r="AG47" s="22"/>
-      <c r="AH47" s="22"/>
-      <c r="AI47" s="22"/>
-      <c r="AJ47" s="22"/>
-      <c r="AK47" s="22"/>
-      <c r="AL47" s="22"/>
-      <c r="AM47" s="22"/>
-      <c r="AN47" s="22"/>
-      <c r="AO47" s="22"/>
-      <c r="AP47" s="22"/>
-      <c r="AQ47" s="22"/>
-      <c r="AR47" s="22"/>
-      <c r="AS47" s="22"/>
-      <c r="AT47" s="22"/>
-      <c r="AU47" s="22"/>
-      <c r="AV47" s="22"/>
-      <c r="AW47" s="22"/>
-      <c r="AX47" s="22"/>
-      <c r="AY47" s="22"/>
-      <c r="AZ47" s="22"/>
-      <c r="BA47" s="22"/>
-      <c r="BB47" s="22"/>
-      <c r="BC47" s="22"/>
-      <c r="BD47" s="22"/>
-      <c r="BE47" s="22"/>
-      <c r="BF47" s="22"/>
-      <c r="BG47" s="22"/>
-      <c r="BH47" s="22"/>
-      <c r="BI47" s="22"/>
-      <c r="BJ47" s="22"/>
-      <c r="BK47" s="22"/>
-    </row>
-    <row r="48" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="25"/>
-      <c r="B48" s="62" t="s">
-        <v>60</v>
-      </c>
-      <c r="C48" s="61"/>
-      <c r="D48" s="63">
-        <f>E47+1</f>
-        <v>46162</v>
-      </c>
-      <c r="E48" s="63">
-        <f>D48+1</f>
-        <v>46163</v>
-      </c>
-      <c r="F48" s="9"/>
-      <c r="G48" s="9"/>
-      <c r="H48" s="22"/>
-      <c r="I48" s="22"/>
-      <c r="J48" s="22"/>
-      <c r="K48" s="22"/>
-      <c r="L48" s="22"/>
-      <c r="M48" s="22"/>
-      <c r="N48" s="22"/>
-      <c r="O48" s="22"/>
-      <c r="P48" s="22"/>
-      <c r="Q48" s="22"/>
-      <c r="R48" s="22"/>
-      <c r="S48" s="22"/>
-      <c r="T48" s="22"/>
-      <c r="U48" s="22"/>
-      <c r="V48" s="22"/>
-      <c r="W48" s="22"/>
-      <c r="X48" s="22"/>
-      <c r="Y48" s="22"/>
-      <c r="Z48" s="22"/>
-      <c r="AA48" s="22"/>
-      <c r="AB48" s="22"/>
-      <c r="AC48" s="22"/>
-      <c r="AD48" s="22"/>
-      <c r="AE48" s="22"/>
-      <c r="AF48" s="22"/>
-      <c r="AG48" s="22"/>
-      <c r="AH48" s="22"/>
-      <c r="AI48" s="22"/>
-      <c r="AJ48" s="22"/>
-      <c r="AK48" s="22"/>
-      <c r="AL48" s="22"/>
-      <c r="AM48" s="22"/>
-      <c r="AN48" s="22"/>
-      <c r="AO48" s="22"/>
-      <c r="AP48" s="22"/>
-      <c r="AQ48" s="22"/>
-      <c r="AR48" s="22"/>
-      <c r="AS48" s="22"/>
-      <c r="AT48" s="22"/>
-      <c r="AU48" s="22"/>
-      <c r="AV48" s="22"/>
-      <c r="AW48" s="22"/>
-      <c r="AX48" s="22"/>
-      <c r="AY48" s="22"/>
-      <c r="AZ48" s="22"/>
-      <c r="BA48" s="22"/>
-      <c r="BB48" s="22"/>
-      <c r="BC48" s="22"/>
-      <c r="BD48" s="22"/>
-      <c r="BE48" s="22"/>
-      <c r="BF48" s="22"/>
-      <c r="BG48" s="22"/>
-      <c r="BH48" s="22"/>
-      <c r="BI48" s="22"/>
-      <c r="BJ48" s="22"/>
-      <c r="BK48" s="22"/>
-    </row>
-    <row r="49" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="25"/>
-      <c r="B49" s="62" t="s">
-        <v>61</v>
-      </c>
-      <c r="C49" s="61"/>
-      <c r="D49" s="63">
-        <f>E48+1</f>
-        <v>46164</v>
-      </c>
-      <c r="E49" s="63">
-        <f>D49+1</f>
-        <v>46165</v>
-      </c>
-      <c r="F49" s="9"/>
-      <c r="G49" s="9"/>
-      <c r="H49" s="22"/>
-      <c r="I49" s="22"/>
-      <c r="J49" s="22"/>
-      <c r="K49" s="22"/>
-      <c r="L49" s="22"/>
-      <c r="M49" s="22"/>
-      <c r="N49" s="22"/>
-      <c r="O49" s="22"/>
-      <c r="P49" s="22"/>
-      <c r="Q49" s="22"/>
-      <c r="R49" s="22"/>
-      <c r="S49" s="22"/>
-      <c r="T49" s="22"/>
-      <c r="U49" s="22"/>
-      <c r="V49" s="22"/>
-      <c r="W49" s="22"/>
-      <c r="X49" s="22"/>
-      <c r="Y49" s="22"/>
-      <c r="Z49" s="22"/>
-      <c r="AA49" s="22"/>
-      <c r="AB49" s="22"/>
-      <c r="AC49" s="22"/>
-      <c r="AD49" s="22"/>
-      <c r="AE49" s="22"/>
-      <c r="AF49" s="22"/>
-      <c r="AG49" s="22"/>
-      <c r="AH49" s="22"/>
-      <c r="AI49" s="22"/>
-      <c r="AJ49" s="22"/>
-      <c r="AK49" s="22"/>
-      <c r="AL49" s="22"/>
-      <c r="AM49" s="22"/>
-      <c r="AN49" s="22"/>
-      <c r="AO49" s="22"/>
-      <c r="AP49" s="22"/>
-      <c r="AQ49" s="22"/>
-      <c r="AR49" s="22"/>
-      <c r="AS49" s="22"/>
-      <c r="AT49" s="22"/>
-      <c r="AU49" s="22"/>
-      <c r="AV49" s="22"/>
-      <c r="AW49" s="22"/>
-      <c r="AX49" s="22"/>
-      <c r="AY49" s="22"/>
-      <c r="AZ49" s="22"/>
-      <c r="BA49" s="22"/>
-      <c r="BB49" s="22"/>
-      <c r="BC49" s="22"/>
-      <c r="BD49" s="22"/>
-      <c r="BE49" s="22"/>
-      <c r="BF49" s="22"/>
-      <c r="BG49" s="22"/>
-      <c r="BH49" s="22"/>
-      <c r="BI49" s="22"/>
-      <c r="BJ49" s="22"/>
-      <c r="BK49" s="22"/>
-    </row>
-    <row r="50" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="25" t="s">
-        <v>18</v>
-      </c>
-      <c r="B50" s="62" t="s">
-        <v>62</v>
-      </c>
-      <c r="C50" s="61"/>
-      <c r="D50" s="63">
-        <f>E49+1</f>
-        <v>46166</v>
-      </c>
-      <c r="E50" s="63">
-        <f>D50+3</f>
-        <v>46169</v>
-      </c>
-      <c r="F50" s="9"/>
-      <c r="G50" s="9">
-        <f t="shared" si="6"/>
-        <v>4</v>
-      </c>
-      <c r="H50" s="22"/>
-      <c r="I50" s="22"/>
-      <c r="J50" s="22"/>
-      <c r="K50" s="22"/>
-      <c r="L50" s="22"/>
-      <c r="M50" s="22"/>
-      <c r="N50" s="22"/>
-      <c r="O50" s="22"/>
-      <c r="P50" s="22"/>
-      <c r="Q50" s="22"/>
-      <c r="R50" s="22"/>
-      <c r="S50" s="22"/>
-      <c r="T50" s="22"/>
-      <c r="U50" s="22"/>
-      <c r="V50" s="22"/>
-      <c r="W50" s="22"/>
-      <c r="X50" s="22"/>
-      <c r="Y50" s="22"/>
-      <c r="Z50" s="22"/>
-      <c r="AA50" s="22"/>
-      <c r="AB50" s="22"/>
-      <c r="AC50" s="22"/>
-      <c r="AD50" s="22"/>
-      <c r="AE50" s="22"/>
-      <c r="AF50" s="22"/>
-      <c r="AG50" s="22"/>
-      <c r="AH50" s="22"/>
-      <c r="AI50" s="22"/>
-      <c r="AJ50" s="22"/>
-      <c r="AK50" s="22"/>
-      <c r="AL50" s="22"/>
-      <c r="AM50" s="22"/>
-      <c r="AN50" s="22"/>
-      <c r="AO50" s="22"/>
-      <c r="AP50" s="22"/>
-      <c r="AQ50" s="22"/>
-      <c r="AR50" s="22"/>
-      <c r="AS50" s="22"/>
-      <c r="AT50" s="22"/>
-      <c r="AU50" s="22"/>
-      <c r="AV50" s="22"/>
-      <c r="AW50" s="22"/>
-      <c r="AX50" s="22"/>
-      <c r="AY50" s="22"/>
-      <c r="AZ50" s="22"/>
-      <c r="BA50" s="22"/>
-      <c r="BB50" s="22"/>
-      <c r="BC50" s="22"/>
-      <c r="BD50" s="22"/>
-      <c r="BE50" s="22"/>
-      <c r="BF50" s="22"/>
-      <c r="BG50" s="22"/>
-      <c r="BH50" s="22"/>
-      <c r="BI50" s="22"/>
-      <c r="BJ50" s="22"/>
-      <c r="BK50" s="22"/>
-    </row>
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="BE4:BK4"/>
@@ -5799,7 +5028,7 @@
     <mergeCell ref="AQ4:AW4"/>
     <mergeCell ref="AX4:BD4"/>
   </mergeCells>
-  <conditionalFormatting sqref="C29:C34 C41:C42 C7:C17">
+  <conditionalFormatting sqref="C30:C33 C7:C18">
     <cfRule type="dataBar" priority="43">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5813,12 +5042,12 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H29:BK49 H5:BK10 H13:BK17 H12:L12 N12:BK12 H11:M11 O11:BK11">
+  <conditionalFormatting sqref="H5:BK10 H13:BK18 H12:L12 N12:BK12 H11:M11 O11:BK11 H30:BK39">
     <cfRule type="expression" dxfId="11" priority="62">
       <formula>AND(TODAY()&gt;=H$5,TODAY()&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H29:BK49 H7:BK10 H13:BK17 H12:L12 N12:BK12 H11:M11 O11:BK11">
+  <conditionalFormatting sqref="H7:BK10 H13:BK18 H12:L12 N12:BK12 H11:M11 O11:BK11 H30:BK39">
     <cfRule type="expression" dxfId="10" priority="56">
       <formula>AND(task_start&lt;=H$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=H$5)</formula>
     </cfRule>
@@ -5826,7 +5055,7 @@
       <formula>AND(task_end&gt;=H$5,task_start&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C18:C19">
+  <conditionalFormatting sqref="C19:C20">
     <cfRule type="dataBar" priority="26">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5840,12 +5069,12 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H18:BK28">
+  <conditionalFormatting sqref="H19:BK29">
     <cfRule type="expression" dxfId="8" priority="29">
       <formula>AND(TODAY()&gt;=H$5,TODAY()&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H18:BK28">
+  <conditionalFormatting sqref="H19:BK29">
     <cfRule type="expression" dxfId="7" priority="27">
       <formula>AND(task_start&lt;=H$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=H$5)</formula>
     </cfRule>
@@ -5853,7 +5082,7 @@
       <formula>AND(task_end&gt;=H$5,task_start&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C20">
+  <conditionalFormatting sqref="C21">
     <cfRule type="dataBar" priority="25">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5867,7 +5096,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C21">
+  <conditionalFormatting sqref="C22">
     <cfRule type="dataBar" priority="24">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5881,7 +5110,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C22">
+  <conditionalFormatting sqref="C23">
     <cfRule type="dataBar" priority="23">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5895,7 +5124,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C23">
+  <conditionalFormatting sqref="C24">
     <cfRule type="dataBar" priority="22">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5909,7 +5138,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C24">
+  <conditionalFormatting sqref="C25">
     <cfRule type="dataBar" priority="21">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5923,7 +5152,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C25">
+  <conditionalFormatting sqref="C26">
     <cfRule type="dataBar" priority="20">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5937,7 +5166,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C26">
+  <conditionalFormatting sqref="C27">
     <cfRule type="dataBar" priority="19">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5951,7 +5180,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C27">
+  <conditionalFormatting sqref="C28">
     <cfRule type="dataBar" priority="18">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5965,7 +5194,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C28">
+  <conditionalFormatting sqref="C29">
     <cfRule type="dataBar" priority="17">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5979,49 +5208,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C35">
-    <cfRule type="dataBar" priority="16">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color theme="0" tint="-0.249977111117893"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2237825B-D0F2-438A-BF7C-77EFBA2A9A82}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C36">
-    <cfRule type="dataBar" priority="15">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color theme="0" tint="-0.249977111117893"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7B2890CC-5659-484F-A743-A4B694B8417F}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C37:C40">
-    <cfRule type="dataBar" priority="14">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color theme="0" tint="-0.249977111117893"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6244F2E6-B093-4685-8806-B6474AF5362C}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C43">
+  <conditionalFormatting sqref="C34">
     <cfRule type="dataBar" priority="9">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -6035,21 +5222,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C44">
-    <cfRule type="dataBar" priority="8">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color theme="0" tint="-0.249977111117893"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0BE3D0F7-4E26-437D-86CD-24DBEBD62166}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C45">
+  <conditionalFormatting sqref="C35">
     <cfRule type="dataBar" priority="7">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -6063,7 +5236,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C50">
+  <conditionalFormatting sqref="C40">
     <cfRule type="dataBar" priority="3">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -6077,12 +5250,12 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H50:BK50">
+  <conditionalFormatting sqref="H40:BK40">
     <cfRule type="expression" dxfId="5" priority="6">
       <formula>AND(TODAY()&gt;=H$5,TODAY()&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H50:BK50">
+  <conditionalFormatting sqref="H40:BK40">
     <cfRule type="expression" dxfId="4" priority="4">
       <formula>AND(task_start&lt;=H$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=H$5)</formula>
     </cfRule>
@@ -6090,7 +5263,7 @@
       <formula>AND(task_end&gt;=H$5,task_start&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C46">
+  <conditionalFormatting sqref="C36">
     <cfRule type="dataBar" priority="2">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -6104,7 +5277,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C47:C49">
+  <conditionalFormatting sqref="C37:C39">
     <cfRule type="dataBar" priority="1">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -6158,7 +5331,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>C29:C34 C41:C42 C7:C17</xm:sqref>
+          <xm:sqref>C30:C33 C7:C18</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{1E90BFA6-AA09-4C84-9DA7-1419DF975915}">
@@ -6173,7 +5346,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>C18:C19</xm:sqref>
+          <xm:sqref>C19:C20</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{8B62DB47-8442-45D6-BEC3-74DDF8582AE9}">
@@ -6188,7 +5361,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>C20</xm:sqref>
+          <xm:sqref>C21</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{16F932DB-37BA-4B6F-B3DA-1BF403ECCAFA}">
@@ -6203,7 +5376,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>C21</xm:sqref>
+          <xm:sqref>C22</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{58D685B9-F45B-4170-8504-C6091E7052FA}">
@@ -6218,7 +5391,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>C22</xm:sqref>
+          <xm:sqref>C23</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{78297278-95C1-42FE-9F04-855A3F8B3896}">
@@ -6233,7 +5406,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>C23</xm:sqref>
+          <xm:sqref>C24</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{C76118F8-2A3A-4C74-B114-7608AE5937D7}">
@@ -6248,7 +5421,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>C24</xm:sqref>
+          <xm:sqref>C25</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{07B4BE8A-B3A4-438A-B4C4-1A17594A88C3}">
@@ -6263,7 +5436,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>C25</xm:sqref>
+          <xm:sqref>C26</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{C18933D9-CEAD-4CCF-BC62-D46734FF5524}">
@@ -6278,7 +5451,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>C26</xm:sqref>
+          <xm:sqref>C27</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{6A65D368-5353-4F64-89E1-0CAA4048C318}">
@@ -6293,7 +5466,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>C27</xm:sqref>
+          <xm:sqref>C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{7FE6434E-EE80-49B2-A22E-A0B943AAD725}">
@@ -6308,10 +5481,25 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>C28</xm:sqref>
+          <xm:sqref>C29</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2237825B-D0F2-438A-BF7C-77EFBA2A9A82}">
+          <x14:cfRule type="dataBar" id="{620CC134-46A1-4F91-A051-9D1345C3FA5D}">
+            <x14:dataBar minLength="0" maxLength="100" gradient="0">
+              <x14:cfvo type="num">
+                <xm:f>0</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="num">
+                <xm:f>1</xm:f>
+              </x14:cfvo>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>C34</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{2CFE5318-DB6A-49E9-A71F-350550A6317A}">
             <x14:dataBar minLength="0" maxLength="100" gradient="0">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -6326,7 +5514,22 @@
           <xm:sqref>C35</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7B2890CC-5659-484F-A743-A4B694B8417F}">
+          <x14:cfRule type="dataBar" id="{4BA551C2-EE6C-4479-BB90-42C647FFB418}">
+            <x14:dataBar minLength="0" maxLength="100" gradient="0">
+              <x14:cfvo type="num">
+                <xm:f>0</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="num">
+                <xm:f>1</xm:f>
+              </x14:cfvo>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>C40</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{06F74896-8DFF-43FC-B666-14565B6A7397}">
             <x14:dataBar minLength="0" maxLength="100" gradient="0">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -6341,96 +5544,6 @@
           <xm:sqref>C36</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6244F2E6-B093-4685-8806-B6474AF5362C}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>1</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>C37:C40</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{620CC134-46A1-4F91-A051-9D1345C3FA5D}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>1</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>C43</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0BE3D0F7-4E26-437D-86CD-24DBEBD62166}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>1</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>C44</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2CFE5318-DB6A-49E9-A71F-350550A6317A}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>1</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>C45</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4BA551C2-EE6C-4479-BB90-42C647FFB418}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>1</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>C50</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{06F74896-8DFF-43FC-B666-14565B6A7397}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>1</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>C46</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{527A852E-2EF7-46F3-8CBA-90E4DD67FCB3}">
             <x14:dataBar minLength="0" maxLength="100" gradient="0">
               <x14:cfvo type="num">
@@ -6443,7 +5556,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>C47:C49</xm:sqref>
+          <xm:sqref>C37:C39</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -6452,6 +5565,35 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Image>
+    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
+    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </ImageTagsTaxHTField>
+    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
+    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="24" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2d714a3296df14eba7a100bb665443ca">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="49549bf45bfbbfb6cffed527380e77e1" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -6739,36 +5881,34 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5144944C-1F1D-4162-962A-96F3FC8455D8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="16c05727-aa75-4e4a-9b5f-8a80a1165891"/>
+    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Image>
-    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
-    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </ImageTagsTaxHTField>
-    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
-    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8FE8ED85-58B3-4608-8E91-0433556D50CE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{708DBB9E-6D89-4A94-9DC5-964B7833E11C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6787,31 +5927,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8FE8ED85-58B3-4608-8E91-0433556D50CE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5144944C-1F1D-4162-962A-96F3FC8455D8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="16c05727-aa75-4e4a-9b5f-8a80a1165891"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualización del listado de requisitos y corrección de variable en la vista de favoritos
</commit_message>
<xml_diff>
--- a/diagramaGANTT.xlsx
+++ b/diagramaGANTT.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{169D5D92-334B-4D19-9601-95BF28CF6789}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4DBF4FC-7EE9-4B78-98FE-CCA15F47D151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="54">
   <si>
     <t>Cree una programación para un proyecto en esta hoja de cálculo.
 Escriba el título de este proyecto en la celda B1. 
@@ -233,6 +233,9 @@
   </si>
   <si>
     <t>Comprar dominio</t>
+  </si>
+  <si>
+    <t>Ranking de zapatillas más favoritas - RFP-017</t>
   </si>
 </sst>
 </file>
@@ -1855,7 +1858,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BK40"/>
+  <dimension ref="A1:BK41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.7109375" style="25" customWidth="1"/>
@@ -2550,7 +2553,7 @@
       <c r="E8" s="38"/>
       <c r="F8" s="9"/>
       <c r="G8" s="9" t="str">
-        <f t="shared" ref="G8:G40" si="6">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+        <f t="shared" ref="G8:G41" si="6">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v/>
       </c>
       <c r="H8" s="22"/>
@@ -3006,7 +3009,7 @@
         <v>1</v>
       </c>
       <c r="D14" s="42">
-        <f t="shared" ref="D14:D29" si="7">E13+1</f>
+        <f t="shared" ref="D14:D30" si="7">E13+1</f>
         <v>46117</v>
       </c>
       <c r="E14" s="42">
@@ -3988,11 +3991,11 @@
     <row r="27" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="25"/>
       <c r="B27" s="31" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C27" s="15"/>
       <c r="D27" s="42">
-        <f t="shared" si="7"/>
+        <f>E26+1</f>
         <v>46136</v>
       </c>
       <c r="E27" s="42">
@@ -4061,16 +4064,16 @@
     <row r="28" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="25"/>
       <c r="B28" s="31" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C28" s="15"/>
       <c r="D28" s="42">
-        <f t="shared" si="7"/>
-        <v>46138</v>
+        <f>E26+1</f>
+        <v>46136</v>
       </c>
       <c r="E28" s="42">
         <f>D28+1</f>
-        <v>46139</v>
+        <v>46137</v>
       </c>
       <c r="F28" s="9"/>
       <c r="G28" s="9"/>
@@ -4134,16 +4137,16 @@
     <row r="29" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="25"/>
       <c r="B29" s="31" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C29" s="15"/>
       <c r="D29" s="42">
-        <f t="shared" si="7"/>
-        <v>46140</v>
+        <f>E28+1</f>
+        <v>46138</v>
       </c>
       <c r="E29" s="42">
-        <f>D29</f>
-        <v>46140</v>
+        <f>D29+1</f>
+        <v>46139</v>
       </c>
       <c r="F29" s="9"/>
       <c r="G29" s="9"/>
@@ -4205,20 +4208,21 @@
       <c r="BK29" s="22"/>
     </row>
     <row r="30" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="25" t="s">
-        <v>18</v>
-      </c>
-      <c r="B30" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="C30" s="17"/>
-      <c r="D30" s="43"/>
-      <c r="E30" s="44"/>
+      <c r="A30" s="25"/>
+      <c r="B30" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="C30" s="15"/>
+      <c r="D30" s="42">
+        <f t="shared" si="7"/>
+        <v>46140</v>
+      </c>
+      <c r="E30" s="42">
+        <f>D30</f>
+        <v>46140</v>
+      </c>
       <c r="F30" s="9"/>
-      <c r="G30" s="9" t="str">
-        <f t="shared" si="6"/>
-        <v/>
-      </c>
+      <c r="G30" s="9"/>
       <c r="H30" s="22"/>
       <c r="I30" s="22"/>
       <c r="J30" s="22"/>
@@ -4277,23 +4281,19 @@
       <c r="BK30" s="22"/>
     </row>
     <row r="31" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="25"/>
-      <c r="B31" s="32" t="s">
-        <v>43</v>
-      </c>
-      <c r="C31" s="18"/>
-      <c r="D31" s="45">
-        <f>E29+1</f>
-        <v>46141</v>
-      </c>
-      <c r="E31" s="45">
-        <f>D31</f>
-        <v>46141</v>
-      </c>
+      <c r="A31" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="B31" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="C31" s="17"/>
+      <c r="D31" s="43"/>
+      <c r="E31" s="44"/>
       <c r="F31" s="9"/>
-      <c r="G31" s="9">
+      <c r="G31" s="9" t="str">
         <f t="shared" si="6"/>
-        <v>1</v>
+        <v/>
       </c>
       <c r="H31" s="22"/>
       <c r="I31" s="22"/>
@@ -4353,19 +4353,23 @@
       <c r="BK31" s="22"/>
     </row>
     <row r="32" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="25" t="s">
-        <v>18</v>
-      </c>
-      <c r="B32" s="19" t="s">
-        <v>44</v>
-      </c>
-      <c r="C32" s="20"/>
-      <c r="D32" s="46"/>
-      <c r="E32" s="47"/>
+      <c r="A32" s="25"/>
+      <c r="B32" s="32" t="s">
+        <v>43</v>
+      </c>
+      <c r="C32" s="18"/>
+      <c r="D32" s="45">
+        <f>E30+1</f>
+        <v>46141</v>
+      </c>
+      <c r="E32" s="45">
+        <f>D32</f>
+        <v>46141</v>
+      </c>
       <c r="F32" s="9"/>
-      <c r="G32" s="9" t="str">
+      <c r="G32" s="9">
         <f t="shared" si="6"/>
-        <v/>
+        <v>1</v>
       </c>
       <c r="H32" s="22"/>
       <c r="I32" s="22"/>
@@ -4425,23 +4429,19 @@
       <c r="BK32" s="22"/>
     </row>
     <row r="33" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="25"/>
-      <c r="B33" s="33" t="s">
-        <v>52</v>
-      </c>
-      <c r="C33" s="21"/>
-      <c r="D33" s="48">
-        <f>E31+1</f>
-        <v>46142</v>
-      </c>
-      <c r="E33" s="48">
-        <f>D33</f>
-        <v>46142</v>
-      </c>
+      <c r="A33" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="B33" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="C33" s="20"/>
+      <c r="D33" s="46"/>
+      <c r="E33" s="47"/>
       <c r="F33" s="9"/>
-      <c r="G33" s="9">
+      <c r="G33" s="9" t="str">
         <f t="shared" si="6"/>
-        <v>1</v>
+        <v/>
       </c>
       <c r="H33" s="22"/>
       <c r="I33" s="22"/>
@@ -4503,21 +4503,21 @@
     <row r="34" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="25"/>
       <c r="B34" s="33" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="C34" s="21"/>
       <c r="D34" s="48">
-        <f>E33+1</f>
-        <v>46143</v>
+        <f>E32+1</f>
+        <v>46142</v>
       </c>
       <c r="E34" s="48">
-        <f>D34+2</f>
-        <v>46145</v>
+        <f>D34</f>
+        <v>46142</v>
       </c>
       <c r="F34" s="9"/>
       <c r="G34" s="9">
         <f t="shared" si="6"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H34" s="22"/>
       <c r="I34" s="22"/>
@@ -4579,21 +4579,21 @@
     <row r="35" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="25"/>
       <c r="B35" s="33" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C35" s="21"/>
       <c r="D35" s="48">
         <f>E34+1</f>
-        <v>46146</v>
+        <v>46143</v>
       </c>
       <c r="E35" s="48">
-        <f>D35</f>
-        <v>46146</v>
+        <f>D35+2</f>
+        <v>46145</v>
       </c>
       <c r="F35" s="9"/>
       <c r="G35" s="9">
         <f t="shared" si="6"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H35" s="22"/>
       <c r="I35" s="22"/>
@@ -4654,14 +4654,23 @@
     </row>
     <row r="36" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="25"/>
-      <c r="B36" s="57" t="s">
-        <v>22</v>
-      </c>
-      <c r="C36" s="58"/>
-      <c r="D36" s="59"/>
-      <c r="E36" s="60"/>
+      <c r="B36" s="33" t="s">
+        <v>46</v>
+      </c>
+      <c r="C36" s="21"/>
+      <c r="D36" s="48">
+        <f>E35+1</f>
+        <v>46146</v>
+      </c>
+      <c r="E36" s="48">
+        <f>D36</f>
+        <v>46146</v>
+      </c>
       <c r="F36" s="9"/>
-      <c r="G36" s="9"/>
+      <c r="G36" s="9">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
       <c r="H36" s="22"/>
       <c r="I36" s="22"/>
       <c r="J36" s="22"/>
@@ -4721,18 +4730,12 @@
     </row>
     <row r="37" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="25"/>
-      <c r="B37" s="62" t="s">
-        <v>47</v>
-      </c>
-      <c r="C37" s="61"/>
-      <c r="D37" s="63">
-        <f>E35+1</f>
-        <v>46147</v>
-      </c>
-      <c r="E37" s="63">
-        <f>D37+1</f>
-        <v>46148</v>
-      </c>
+      <c r="B37" s="57" t="s">
+        <v>22</v>
+      </c>
+      <c r="C37" s="58"/>
+      <c r="D37" s="59"/>
+      <c r="E37" s="60"/>
       <c r="F37" s="9"/>
       <c r="G37" s="9"/>
       <c r="H37" s="22"/>
@@ -4795,16 +4798,16 @@
     <row r="38" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="25"/>
       <c r="B38" s="62" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C38" s="61"/>
       <c r="D38" s="63">
-        <f>E37+1</f>
-        <v>46149</v>
+        <f>E36+1</f>
+        <v>46147</v>
       </c>
       <c r="E38" s="63">
         <f>D38+1</f>
-        <v>46150</v>
+        <v>46148</v>
       </c>
       <c r="F38" s="9"/>
       <c r="G38" s="9"/>
@@ -4868,16 +4871,16 @@
     <row r="39" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="25"/>
       <c r="B39" s="62" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C39" s="61"/>
       <c r="D39" s="63">
         <f>E38+1</f>
-        <v>46151</v>
+        <v>46149</v>
       </c>
       <c r="E39" s="63">
         <f>D39+1</f>
-        <v>46152</v>
+        <v>46150</v>
       </c>
       <c r="F39" s="9"/>
       <c r="G39" s="9"/>
@@ -4939,26 +4942,21 @@
       <c r="BK39" s="22"/>
     </row>
     <row r="40" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="25" t="s">
-        <v>18</v>
-      </c>
+      <c r="A40" s="25"/>
       <c r="B40" s="62" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C40" s="61"/>
       <c r="D40" s="63">
         <f>E39+1</f>
-        <v>46153</v>
+        <v>46151</v>
       </c>
       <c r="E40" s="63">
-        <f>D40+3</f>
-        <v>46156</v>
+        <f>D40+1</f>
+        <v>46152</v>
       </c>
       <c r="F40" s="9"/>
-      <c r="G40" s="9">
-        <f t="shared" si="6"/>
-        <v>4</v>
-      </c>
+      <c r="G40" s="9"/>
       <c r="H40" s="22"/>
       <c r="I40" s="22"/>
       <c r="J40" s="22"/>
@@ -5016,6 +5014,84 @@
       <c r="BJ40" s="22"/>
       <c r="BK40" s="22"/>
     </row>
+    <row r="41" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="B41" s="62" t="s">
+        <v>50</v>
+      </c>
+      <c r="C41" s="61"/>
+      <c r="D41" s="63">
+        <f>E40+1</f>
+        <v>46153</v>
+      </c>
+      <c r="E41" s="63">
+        <f>D41+3</f>
+        <v>46156</v>
+      </c>
+      <c r="F41" s="9"/>
+      <c r="G41" s="9">
+        <f t="shared" si="6"/>
+        <v>4</v>
+      </c>
+      <c r="H41" s="22"/>
+      <c r="I41" s="22"/>
+      <c r="J41" s="22"/>
+      <c r="K41" s="22"/>
+      <c r="L41" s="22"/>
+      <c r="M41" s="22"/>
+      <c r="N41" s="22"/>
+      <c r="O41" s="22"/>
+      <c r="P41" s="22"/>
+      <c r="Q41" s="22"/>
+      <c r="R41" s="22"/>
+      <c r="S41" s="22"/>
+      <c r="T41" s="22"/>
+      <c r="U41" s="22"/>
+      <c r="V41" s="22"/>
+      <c r="W41" s="22"/>
+      <c r="X41" s="22"/>
+      <c r="Y41" s="22"/>
+      <c r="Z41" s="22"/>
+      <c r="AA41" s="22"/>
+      <c r="AB41" s="22"/>
+      <c r="AC41" s="22"/>
+      <c r="AD41" s="22"/>
+      <c r="AE41" s="22"/>
+      <c r="AF41" s="22"/>
+      <c r="AG41" s="22"/>
+      <c r="AH41" s="22"/>
+      <c r="AI41" s="22"/>
+      <c r="AJ41" s="22"/>
+      <c r="AK41" s="22"/>
+      <c r="AL41" s="22"/>
+      <c r="AM41" s="22"/>
+      <c r="AN41" s="22"/>
+      <c r="AO41" s="22"/>
+      <c r="AP41" s="22"/>
+      <c r="AQ41" s="22"/>
+      <c r="AR41" s="22"/>
+      <c r="AS41" s="22"/>
+      <c r="AT41" s="22"/>
+      <c r="AU41" s="22"/>
+      <c r="AV41" s="22"/>
+      <c r="AW41" s="22"/>
+      <c r="AX41" s="22"/>
+      <c r="AY41" s="22"/>
+      <c r="AZ41" s="22"/>
+      <c r="BA41" s="22"/>
+      <c r="BB41" s="22"/>
+      <c r="BC41" s="22"/>
+      <c r="BD41" s="22"/>
+      <c r="BE41" s="22"/>
+      <c r="BF41" s="22"/>
+      <c r="BG41" s="22"/>
+      <c r="BH41" s="22"/>
+      <c r="BI41" s="22"/>
+      <c r="BJ41" s="22"/>
+      <c r="BK41" s="22"/>
+    </row>
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="BE4:BK4"/>
@@ -5028,7 +5104,7 @@
     <mergeCell ref="AQ4:AW4"/>
     <mergeCell ref="AX4:BD4"/>
   </mergeCells>
-  <conditionalFormatting sqref="C30:C33 C7:C18">
+  <conditionalFormatting sqref="C31:C34 C7:C18">
     <cfRule type="dataBar" priority="43">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5042,12 +5118,12 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H5:BK10 H13:BK18 H12:L12 N12:BK12 H11:M11 O11:BK11 H30:BK39">
+  <conditionalFormatting sqref="H5:BK10 H13:BK18 H12:L12 N12:BK12 H11:M11 O11:BK11 H31:BK40">
     <cfRule type="expression" dxfId="11" priority="62">
       <formula>AND(TODAY()&gt;=H$5,TODAY()&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H7:BK10 H13:BK18 H12:L12 N12:BK12 H11:M11 O11:BK11 H30:BK39">
+  <conditionalFormatting sqref="H7:BK10 H13:BK18 H12:L12 N12:BK12 H11:M11 O11:BK11 H31:BK40">
     <cfRule type="expression" dxfId="10" priority="56">
       <formula>AND(task_start&lt;=H$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=H$5)</formula>
     </cfRule>
@@ -5069,12 +5145,12 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H19:BK29">
+  <conditionalFormatting sqref="H19:BK30">
     <cfRule type="expression" dxfId="8" priority="29">
       <formula>AND(TODAY()&gt;=H$5,TODAY()&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H19:BK29">
+  <conditionalFormatting sqref="H19:BK30">
     <cfRule type="expression" dxfId="7" priority="27">
       <formula>AND(task_start&lt;=H$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=H$5)</formula>
     </cfRule>
@@ -5152,7 +5228,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C26">
+  <conditionalFormatting sqref="C26:C27">
     <cfRule type="dataBar" priority="20">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5166,7 +5242,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C27">
+  <conditionalFormatting sqref="C28">
     <cfRule type="dataBar" priority="19">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5180,7 +5256,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C28">
+  <conditionalFormatting sqref="C29">
     <cfRule type="dataBar" priority="18">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5194,7 +5270,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C29">
+  <conditionalFormatting sqref="C30">
     <cfRule type="dataBar" priority="17">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5208,7 +5284,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C34">
+  <conditionalFormatting sqref="C35">
     <cfRule type="dataBar" priority="9">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5222,7 +5298,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C35">
+  <conditionalFormatting sqref="C36">
     <cfRule type="dataBar" priority="7">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5236,7 +5312,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C40">
+  <conditionalFormatting sqref="C41">
     <cfRule type="dataBar" priority="3">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5250,12 +5326,12 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H40:BK40">
+  <conditionalFormatting sqref="H41:BK41">
     <cfRule type="expression" dxfId="5" priority="6">
       <formula>AND(TODAY()&gt;=H$5,TODAY()&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H40:BK40">
+  <conditionalFormatting sqref="H41:BK41">
     <cfRule type="expression" dxfId="4" priority="4">
       <formula>AND(task_start&lt;=H$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=H$5)</formula>
     </cfRule>
@@ -5263,7 +5339,7 @@
       <formula>AND(task_end&gt;=H$5,task_start&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C36">
+  <conditionalFormatting sqref="C37">
     <cfRule type="dataBar" priority="2">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5277,7 +5353,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C37:C39">
+  <conditionalFormatting sqref="C38:C40">
     <cfRule type="dataBar" priority="1">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5331,7 +5407,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>C30:C33 C7:C18</xm:sqref>
+          <xm:sqref>C31:C34 C7:C18</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{1E90BFA6-AA09-4C84-9DA7-1419DF975915}">
@@ -5436,7 +5512,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>C26</xm:sqref>
+          <xm:sqref>C26:C27</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{C18933D9-CEAD-4CCF-BC62-D46734FF5524}">
@@ -5451,7 +5527,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>C27</xm:sqref>
+          <xm:sqref>C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{6A65D368-5353-4F64-89E1-0CAA4048C318}">
@@ -5466,7 +5542,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>C28</xm:sqref>
+          <xm:sqref>C29</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{7FE6434E-EE80-49B2-A22E-A0B943AAD725}">
@@ -5481,7 +5557,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>C29</xm:sqref>
+          <xm:sqref>C30</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{620CC134-46A1-4F91-A051-9D1345C3FA5D}">
@@ -5496,7 +5572,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>C34</xm:sqref>
+          <xm:sqref>C35</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{2CFE5318-DB6A-49E9-A71F-350550A6317A}">
@@ -5511,7 +5587,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>C35</xm:sqref>
+          <xm:sqref>C36</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{4BA551C2-EE6C-4479-BB90-42C647FFB418}">
@@ -5526,7 +5602,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>C40</xm:sqref>
+          <xm:sqref>C41</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{06F74896-8DFF-43FC-B666-14565B6A7397}">
@@ -5541,7 +5617,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>C36</xm:sqref>
+          <xm:sqref>C37</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{527A852E-2EF7-46F3-8CBA-90E4DD67FCB3}">
@@ -5556,7 +5632,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>C37:C39</xm:sqref>
+          <xm:sqref>C38:C40</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -5565,35 +5641,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Image>
-    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
-    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </ImageTagsTaxHTField>
-    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
-    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="24" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2d714a3296df14eba7a100bb665443ca">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="49549bf45bfbbfb6cffed527380e77e1" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -5881,34 +5928,36 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5144944C-1F1D-4162-962A-96F3FC8455D8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="16c05727-aa75-4e4a-9b5f-8a80a1165891"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8FE8ED85-58B3-4608-8E91-0433556D50CE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Image>
+    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
+    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </ImageTagsTaxHTField>
+    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
+    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{708DBB9E-6D89-4A94-9DC5-964B7833E11C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5927,4 +5976,31 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8FE8ED85-58B3-4608-8E91-0433556D50CE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5144944C-1F1D-4162-962A-96F3FC8455D8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="16c05727-aa75-4e4a-9b5f-8a80a1165891"/>
+    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizar diagrama GANTT con nuevas modificaciones
</commit_message>
<xml_diff>
--- a/diagramaGANTT.xlsx
+++ b/diagramaGANTT.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4DBF4FC-7EE9-4B78-98FE-CCA15F47D151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49D02353-0A08-46CE-9663-6F0A41872B58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3778,7 +3778,7 @@
         <v>46132</v>
       </c>
       <c r="E24" s="42">
-        <f>D24+1</f>
+        <f t="shared" ref="E24:E29" si="8">D24+1</f>
         <v>46133</v>
       </c>
       <c r="F24" s="9"/>
@@ -3853,7 +3853,7 @@
         <v>46132</v>
       </c>
       <c r="E25" s="42">
-        <f>D25+1</f>
+        <f t="shared" si="8"/>
         <v>46133</v>
       </c>
       <c r="F25" s="9"/>
@@ -3920,13 +3920,15 @@
       <c r="B26" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="C26" s="15"/>
+      <c r="C26" s="15">
+        <v>1</v>
+      </c>
       <c r="D26" s="42">
         <f t="shared" si="7"/>
         <v>46134</v>
       </c>
       <c r="E26" s="42">
-        <f>D26+1</f>
+        <f t="shared" si="8"/>
         <v>46135</v>
       </c>
       <c r="F26" s="9"/>
@@ -3999,7 +4001,7 @@
         <v>46136</v>
       </c>
       <c r="E27" s="42">
-        <f>D27+1</f>
+        <f t="shared" si="8"/>
         <v>46137</v>
       </c>
       <c r="F27" s="9"/>
@@ -4072,7 +4074,7 @@
         <v>46136</v>
       </c>
       <c r="E28" s="42">
-        <f>D28+1</f>
+        <f t="shared" si="8"/>
         <v>46137</v>
       </c>
       <c r="F28" s="9"/>
@@ -4145,7 +4147,7 @@
         <v>46138</v>
       </c>
       <c r="E29" s="42">
-        <f>D29+1</f>
+        <f t="shared" si="8"/>
         <v>46139</v>
       </c>
       <c r="F29" s="9"/>
@@ -5641,6 +5643,35 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Image>
+    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
+    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </ImageTagsTaxHTField>
+    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
+    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="24" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2d714a3296df14eba7a100bb665443ca">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="49549bf45bfbbfb6cffed527380e77e1" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -5928,36 +5959,34 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5144944C-1F1D-4162-962A-96F3FC8455D8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="16c05727-aa75-4e4a-9b5f-8a80a1165891"/>
+    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Image>
-    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
-    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </ImageTagsTaxHTField>
-    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
-    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8FE8ED85-58B3-4608-8E91-0433556D50CE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{708DBB9E-6D89-4A94-9DC5-964B7833E11C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5976,31 +6005,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8FE8ED85-58B3-4608-8E91-0433556D50CE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5144944C-1F1D-4162-962A-96F3FC8455D8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="16c05727-aa75-4e4a-9b5f-8a80a1165891"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Eliminar mensajes de sesión innecesarios en varias vistas
</commit_message>
<xml_diff>
--- a/diagramaGANTT.xlsx
+++ b/diagramaGANTT.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C879E7F4-FAE3-44D8-99DC-3FFB5E28F140}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAAC041D-A602-4BA0-94EE-6448D51C1CCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3995,7 +3995,9 @@
       <c r="B27" s="31" t="s">
         <v>52</v>
       </c>
-      <c r="C27" s="15"/>
+      <c r="C27" s="15">
+        <v>1</v>
+      </c>
       <c r="D27" s="42">
         <f>E26+1</f>
         <v>46136</v>
@@ -5645,6 +5647,35 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Image>
+    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
+    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </ImageTagsTaxHTField>
+    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
+    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="24" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2d714a3296df14eba7a100bb665443ca">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="49549bf45bfbbfb6cffed527380e77e1" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -5932,36 +5963,34 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5144944C-1F1D-4162-962A-96F3FC8455D8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="16c05727-aa75-4e4a-9b5f-8a80a1165891"/>
+    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Image>
-    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
-    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </ImageTagsTaxHTField>
-    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
-    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8FE8ED85-58B3-4608-8E91-0433556D50CE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{708DBB9E-6D89-4A94-9DC5-964B7833E11C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5980,31 +6009,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8FE8ED85-58B3-4608-8E91-0433556D50CE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5144944C-1F1D-4162-962A-96F3FC8455D8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="16c05727-aa75-4e4a-9b5f-8a80a1165891"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Mejorar la responsividad del diseño y ajustar estilos en las vistas de zapatillas
</commit_message>
<xml_diff>
--- a/diagramaGANTT.xlsx
+++ b/diagramaGANTT.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAAC041D-A602-4BA0-94EE-6448D51C1CCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8A92CDD-656B-4356-9DFA-867E9FEFED2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4070,7 +4070,9 @@
       <c r="B28" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="C28" s="15"/>
+      <c r="C28" s="15">
+        <v>0</v>
+      </c>
       <c r="D28" s="42">
         <f>E26+1</f>
         <v>46136</v>

</xml_diff>

<commit_message>
Implementar selector de idiomas y mejoras de traducciones en las vistas, middleware de locale y archivos JSON para soporte bilingüe
</commit_message>
<xml_diff>
--- a/diagramaGANTT.xlsx
+++ b/diagramaGANTT.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8A92CDD-656B-4356-9DFA-867E9FEFED2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5456C15-E78A-42EC-AF72-D51785A33E1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4145,7 +4145,9 @@
       <c r="B29" s="31" t="s">
         <v>41</v>
       </c>
-      <c r="C29" s="15"/>
+      <c r="C29" s="15">
+        <v>1</v>
+      </c>
       <c r="D29" s="42">
         <f>E28+1</f>
         <v>46138</v>
@@ -4218,7 +4220,9 @@
       <c r="B30" s="31" t="s">
         <v>42</v>
       </c>
-      <c r="C30" s="15"/>
+      <c r="C30" s="15">
+        <v>1</v>
+      </c>
       <c r="D30" s="42">
         <f t="shared" si="7"/>
         <v>46140</v>
@@ -4363,7 +4367,9 @@
       <c r="B32" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="C32" s="18"/>
+      <c r="C32" s="18">
+        <v>1</v>
+      </c>
       <c r="D32" s="45">
         <f>E30+1</f>
         <v>46141</v>

</xml_diff>

<commit_message>
Optimizaciones SEO y rendimiento: logo WebP, preload CSS, meta description, accesibilidad, cache Nginx
</commit_message>
<xml_diff>
--- a/diagramaGANTT.xlsx
+++ b/diagramaGANTT.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5456C15-E78A-42EC-AF72-D51785A33E1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7279F0F6-7044-4A41-BAB7-3680584C09A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="52">
   <si>
     <t>Cree una programación para un proyecto en esta hoja de cálculo.
 Escriba el título de este proyecto en la celda B1. 
@@ -214,15 +214,6 @@
     <t>Probar que la web online funciona</t>
   </si>
   <si>
-    <t>Documentación técnica</t>
-  </si>
-  <si>
-    <t>Documentación de usuario</t>
-  </si>
-  <si>
-    <t>Documentación de despliegue</t>
-  </si>
-  <si>
     <t>Entrega final</t>
   </si>
   <si>
@@ -236,6 +227,9 @@
   </si>
   <si>
     <t>Configurar mini pc con web</t>
+  </si>
+  <si>
+    <t>Documentación</t>
   </si>
 </sst>
 </file>
@@ -1021,7 +1015,7 @@
     <xf numFmtId="0" fontId="6" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1201,9 +1195,6 @@
     </xf>
     <xf numFmtId="166" fontId="6" fillId="45" borderId="2" xfId="10" applyFill="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="169" fontId="0" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -1274,37 +1265,7 @@
     <cellStyle name="Total" xfId="29" builtinId="25" customBuiltin="1"/>
     <cellStyle name="zTextoOculto" xfId="3" xr:uid="{26E66EE6-E33F-4D77-BAE4-0FB4F5BBF673}"/>
   </cellStyles>
-  <dxfs count="21">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.34998626667073579"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FFC00000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFC00000"/>
-        </right>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
+  <dxfs count="18">
     <dxf>
       <fill>
         <patternFill>
@@ -1491,15 +1452,15 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="ListaTareasPendientes" pivot="0" count="9" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" dxfId="20"/>
-      <tableStyleElement type="headerRow" dxfId="19"/>
-      <tableStyleElement type="totalRow" dxfId="18"/>
-      <tableStyleElement type="firstColumn" dxfId="17"/>
-      <tableStyleElement type="lastColumn" dxfId="16"/>
-      <tableStyleElement type="firstRowStripe" dxfId="15"/>
-      <tableStyleElement type="secondRowStripe" dxfId="14"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
-      <tableStyleElement type="secondColumnStripe" dxfId="12"/>
+      <tableStyleElement type="wholeTable" dxfId="17"/>
+      <tableStyleElement type="headerRow" dxfId="16"/>
+      <tableStyleElement type="totalRow" dxfId="15"/>
+      <tableStyleElement type="firstColumn" dxfId="14"/>
+      <tableStyleElement type="lastColumn" dxfId="13"/>
+      <tableStyleElement type="firstRowStripe" dxfId="12"/>
+      <tableStyleElement type="secondRowStripe" dxfId="11"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="10"/>
+      <tableStyleElement type="secondColumnStripe" dxfId="9"/>
     </tableStyle>
   </tableStyles>
   <colors>
@@ -1858,7 +1819,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BK41"/>
+  <dimension ref="A1:BD39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.7109375" style="25" customWidth="1"/>
@@ -1868,11 +1829,11 @@
     <col min="5" max="5" width="10.42578125" customWidth="1"/>
     <col min="6" max="6" width="3.140625" customWidth="1"/>
     <col min="7" max="7" width="6.140625" hidden="1" customWidth="1"/>
-    <col min="8" max="63" width="4.7109375" customWidth="1"/>
-    <col min="68" max="69" width="10.28515625"/>
+    <col min="8" max="56" width="4.7109375" customWidth="1"/>
+    <col min="61" max="62" width="10.28515625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:63" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:56" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
@@ -1885,7 +1846,7 @@
       <c r="G1" s="1"/>
       <c r="H1" s="35"/>
     </row>
-    <row r="2" spans="1:63" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:56" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="25" t="s">
         <v>1</v>
       </c>
@@ -1894,7 +1855,7 @@
       </c>
       <c r="H2" s="36"/>
     </row>
-    <row r="3" spans="1:63" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:56" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="25" t="s">
         <v>3</v>
       </c>
@@ -1902,12 +1863,12 @@
         <v>4</v>
       </c>
       <c r="C3" s="52"/>
-      <c r="D3" s="68">
+      <c r="D3" s="67">
         <v>46113</v>
       </c>
-      <c r="E3" s="68"/>
+      <c r="E3" s="67"/>
     </row>
-    <row r="4" spans="1:63" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:56" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="26" t="s">
         <v>5</v>
       </c>
@@ -1915,88 +1876,78 @@
       <c r="D4" s="5">
         <v>1</v>
       </c>
-      <c r="H4" s="65">
+      <c r="H4" s="64">
         <f>H5</f>
         <v>46111</v>
       </c>
-      <c r="I4" s="66"/>
-      <c r="J4" s="66"/>
-      <c r="K4" s="66"/>
-      <c r="L4" s="66"/>
-      <c r="M4" s="66"/>
-      <c r="N4" s="67"/>
-      <c r="O4" s="65">
+      <c r="I4" s="65"/>
+      <c r="J4" s="65"/>
+      <c r="K4" s="65"/>
+      <c r="L4" s="65"/>
+      <c r="M4" s="65"/>
+      <c r="N4" s="66"/>
+      <c r="O4" s="64">
         <f>O5</f>
         <v>46118</v>
       </c>
-      <c r="P4" s="66"/>
-      <c r="Q4" s="66"/>
-      <c r="R4" s="66"/>
-      <c r="S4" s="66"/>
-      <c r="T4" s="66"/>
-      <c r="U4" s="67"/>
-      <c r="V4" s="65">
+      <c r="P4" s="65"/>
+      <c r="Q4" s="65"/>
+      <c r="R4" s="65"/>
+      <c r="S4" s="65"/>
+      <c r="T4" s="65"/>
+      <c r="U4" s="66"/>
+      <c r="V4" s="64">
         <f>V5</f>
         <v>46125</v>
       </c>
-      <c r="W4" s="66"/>
-      <c r="X4" s="66"/>
-      <c r="Y4" s="66"/>
-      <c r="Z4" s="66"/>
-      <c r="AA4" s="66"/>
-      <c r="AB4" s="67"/>
-      <c r="AC4" s="65">
+      <c r="W4" s="65"/>
+      <c r="X4" s="65"/>
+      <c r="Y4" s="65"/>
+      <c r="Z4" s="65"/>
+      <c r="AA4" s="65"/>
+      <c r="AB4" s="66"/>
+      <c r="AC4" s="64">
         <f>AC5</f>
         <v>46132</v>
       </c>
-      <c r="AD4" s="66"/>
-      <c r="AE4" s="66"/>
-      <c r="AF4" s="66"/>
-      <c r="AG4" s="66"/>
-      <c r="AH4" s="66"/>
-      <c r="AI4" s="67"/>
-      <c r="AJ4" s="65">
+      <c r="AD4" s="65"/>
+      <c r="AE4" s="65"/>
+      <c r="AF4" s="65"/>
+      <c r="AG4" s="65"/>
+      <c r="AH4" s="65"/>
+      <c r="AI4" s="66"/>
+      <c r="AJ4" s="64">
         <f>AJ5</f>
         <v>46139</v>
       </c>
-      <c r="AK4" s="66"/>
-      <c r="AL4" s="66"/>
-      <c r="AM4" s="66"/>
-      <c r="AN4" s="66"/>
-      <c r="AO4" s="66"/>
-      <c r="AP4" s="67"/>
-      <c r="AQ4" s="65">
+      <c r="AK4" s="65"/>
+      <c r="AL4" s="65"/>
+      <c r="AM4" s="65"/>
+      <c r="AN4" s="65"/>
+      <c r="AO4" s="65"/>
+      <c r="AP4" s="66"/>
+      <c r="AQ4" s="64">
         <f>AQ5</f>
         <v>46146</v>
       </c>
-      <c r="AR4" s="66"/>
-      <c r="AS4" s="66"/>
-      <c r="AT4" s="66"/>
-      <c r="AU4" s="66"/>
-      <c r="AV4" s="66"/>
-      <c r="AW4" s="67"/>
-      <c r="AX4" s="65">
+      <c r="AR4" s="65"/>
+      <c r="AS4" s="65"/>
+      <c r="AT4" s="65"/>
+      <c r="AU4" s="65"/>
+      <c r="AV4" s="65"/>
+      <c r="AW4" s="66"/>
+      <c r="AX4" s="64">
         <f>AX5</f>
         <v>46153</v>
       </c>
-      <c r="AY4" s="66"/>
-      <c r="AZ4" s="66"/>
-      <c r="BA4" s="66"/>
-      <c r="BB4" s="66"/>
-      <c r="BC4" s="66"/>
-      <c r="BD4" s="67"/>
-      <c r="BE4" s="65">
-        <f>BE5</f>
-        <v>46160</v>
-      </c>
-      <c r="BF4" s="66"/>
-      <c r="BG4" s="66"/>
-      <c r="BH4" s="66"/>
-      <c r="BI4" s="66"/>
-      <c r="BJ4" s="66"/>
-      <c r="BK4" s="67"/>
+      <c r="AY4" s="65"/>
+      <c r="AZ4" s="65"/>
+      <c r="BA4" s="65"/>
+      <c r="BB4" s="65"/>
+      <c r="BC4" s="65"/>
+      <c r="BD4" s="66"/>
     </row>
-    <row r="5" spans="1:63" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:56" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="26" t="s">
         <v>6</v>
       </c>
@@ -2201,36 +2152,8 @@
         <f t="shared" si="1"/>
         <v>46159</v>
       </c>
-      <c r="BE5" s="49">
-        <f>BD5+1</f>
-        <v>46160</v>
-      </c>
-      <c r="BF5" s="50">
-        <f>BE5+1</f>
-        <v>46161</v>
-      </c>
-      <c r="BG5" s="50">
-        <f t="shared" ref="BG5:BK5" si="2">BF5+1</f>
-        <v>46162</v>
-      </c>
-      <c r="BH5" s="50">
-        <f t="shared" si="2"/>
-        <v>46163</v>
-      </c>
-      <c r="BI5" s="50">
-        <f t="shared" si="2"/>
-        <v>46164</v>
-      </c>
-      <c r="BJ5" s="50">
-        <f t="shared" si="2"/>
-        <v>46165</v>
-      </c>
-      <c r="BK5" s="51">
-        <f t="shared" si="2"/>
-        <v>46166</v>
-      </c>
     </row>
-    <row r="6" spans="1:63" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:56" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="26" t="s">
         <v>7</v>
       </c>
@@ -2251,87 +2174,87 @@
         <v>12</v>
       </c>
       <c r="H6" s="8" t="str">
-        <f t="shared" ref="H6" si="3">LEFT(TEXT(H5,"ddd"),1)</f>
+        <f t="shared" ref="H6" si="2">LEFT(TEXT(H5,"ddd"),1)</f>
         <v>l</v>
       </c>
       <c r="I6" s="8" t="str">
-        <f t="shared" ref="I6:AQ6" si="4">LEFT(TEXT(I5,"ddd"),1)</f>
+        <f t="shared" ref="I6:AQ6" si="3">LEFT(TEXT(I5,"ddd"),1)</f>
         <v>m</v>
       </c>
       <c r="J6" s="8" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>m</v>
       </c>
       <c r="K6" s="8" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>j</v>
       </c>
       <c r="L6" s="8" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>v</v>
       </c>
       <c r="M6" s="8" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>s</v>
       </c>
       <c r="N6" s="8" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>d</v>
       </c>
       <c r="O6" s="8" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>l</v>
       </c>
       <c r="P6" s="8" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>m</v>
       </c>
       <c r="Q6" s="8" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>m</v>
       </c>
       <c r="R6" s="8" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>j</v>
       </c>
       <c r="S6" s="8" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>v</v>
       </c>
       <c r="T6" s="8" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>s</v>
       </c>
       <c r="U6" s="8" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>d</v>
       </c>
       <c r="V6" s="8" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>l</v>
       </c>
       <c r="W6" s="8" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>m</v>
       </c>
       <c r="X6" s="8" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>m</v>
       </c>
       <c r="Y6" s="8" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>j</v>
       </c>
       <c r="Z6" s="8" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>v</v>
       </c>
       <c r="AA6" s="8" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>s</v>
       </c>
       <c r="AB6" s="8" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>d</v>
       </c>
       <c r="AC6" s="8" t="str">
@@ -2339,143 +2262,115 @@
         <v>l</v>
       </c>
       <c r="AD6" s="8" t="str">
+        <f t="shared" si="3"/>
+        <v>m</v>
+      </c>
+      <c r="AE6" s="8" t="str">
+        <f t="shared" si="3"/>
+        <v>m</v>
+      </c>
+      <c r="AF6" s="8" t="str">
+        <f t="shared" si="3"/>
+        <v>j</v>
+      </c>
+      <c r="AG6" s="8" t="str">
+        <f t="shared" si="3"/>
+        <v>v</v>
+      </c>
+      <c r="AH6" s="8" t="str">
+        <f t="shared" si="3"/>
+        <v>s</v>
+      </c>
+      <c r="AI6" s="8" t="str">
+        <f t="shared" si="3"/>
+        <v>d</v>
+      </c>
+      <c r="AJ6" s="8" t="str">
+        <f t="shared" si="3"/>
+        <v>l</v>
+      </c>
+      <c r="AK6" s="8" t="str">
+        <f t="shared" si="3"/>
+        <v>m</v>
+      </c>
+      <c r="AL6" s="8" t="str">
+        <f t="shared" si="3"/>
+        <v>m</v>
+      </c>
+      <c r="AM6" s="8" t="str">
+        <f t="shared" si="3"/>
+        <v>j</v>
+      </c>
+      <c r="AN6" s="8" t="str">
+        <f t="shared" si="3"/>
+        <v>v</v>
+      </c>
+      <c r="AO6" s="8" t="str">
+        <f t="shared" si="3"/>
+        <v>s</v>
+      </c>
+      <c r="AP6" s="8" t="str">
+        <f t="shared" si="3"/>
+        <v>d</v>
+      </c>
+      <c r="AQ6" s="8" t="str">
+        <f t="shared" si="3"/>
+        <v>l</v>
+      </c>
+      <c r="AR6" s="8" t="str">
+        <f t="shared" ref="AR6:BD6" si="4">LEFT(TEXT(AR5,"ddd"),1)</f>
+        <v>m</v>
+      </c>
+      <c r="AS6" s="8" t="str">
         <f t="shared" si="4"/>
         <v>m</v>
       </c>
-      <c r="AE6" s="8" t="str">
+      <c r="AT6" s="8" t="str">
+        <f t="shared" si="4"/>
+        <v>j</v>
+      </c>
+      <c r="AU6" s="8" t="str">
+        <f t="shared" si="4"/>
+        <v>v</v>
+      </c>
+      <c r="AV6" s="8" t="str">
+        <f t="shared" si="4"/>
+        <v>s</v>
+      </c>
+      <c r="AW6" s="8" t="str">
+        <f t="shared" si="4"/>
+        <v>d</v>
+      </c>
+      <c r="AX6" s="8" t="str">
+        <f t="shared" si="4"/>
+        <v>l</v>
+      </c>
+      <c r="AY6" s="8" t="str">
         <f t="shared" si="4"/>
         <v>m</v>
       </c>
-      <c r="AF6" s="8" t="str">
+      <c r="AZ6" s="8" t="str">
+        <f t="shared" si="4"/>
+        <v>m</v>
+      </c>
+      <c r="BA6" s="8" t="str">
         <f t="shared" si="4"/>
         <v>j</v>
       </c>
-      <c r="AG6" s="8" t="str">
+      <c r="BB6" s="8" t="str">
         <f t="shared" si="4"/>
         <v>v</v>
       </c>
-      <c r="AH6" s="8" t="str">
+      <c r="BC6" s="8" t="str">
         <f t="shared" si="4"/>
         <v>s</v>
       </c>
-      <c r="AI6" s="8" t="str">
+      <c r="BD6" s="8" t="str">
         <f t="shared" si="4"/>
         <v>d</v>
       </c>
-      <c r="AJ6" s="8" t="str">
-        <f t="shared" si="4"/>
-        <v>l</v>
-      </c>
-      <c r="AK6" s="8" t="str">
-        <f t="shared" si="4"/>
-        <v>m</v>
-      </c>
-      <c r="AL6" s="8" t="str">
-        <f t="shared" si="4"/>
-        <v>m</v>
-      </c>
-      <c r="AM6" s="8" t="str">
-        <f t="shared" si="4"/>
-        <v>j</v>
-      </c>
-      <c r="AN6" s="8" t="str">
-        <f t="shared" si="4"/>
-        <v>v</v>
-      </c>
-      <c r="AO6" s="8" t="str">
-        <f t="shared" si="4"/>
-        <v>s</v>
-      </c>
-      <c r="AP6" s="8" t="str">
-        <f t="shared" si="4"/>
-        <v>d</v>
-      </c>
-      <c r="AQ6" s="8" t="str">
-        <f t="shared" si="4"/>
-        <v>l</v>
-      </c>
-      <c r="AR6" s="8" t="str">
-        <f t="shared" ref="AR6:BK6" si="5">LEFT(TEXT(AR5,"ddd"),1)</f>
-        <v>m</v>
-      </c>
-      <c r="AS6" s="8" t="str">
-        <f t="shared" si="5"/>
-        <v>m</v>
-      </c>
-      <c r="AT6" s="8" t="str">
-        <f t="shared" si="5"/>
-        <v>j</v>
-      </c>
-      <c r="AU6" s="8" t="str">
-        <f t="shared" si="5"/>
-        <v>v</v>
-      </c>
-      <c r="AV6" s="8" t="str">
-        <f t="shared" si="5"/>
-        <v>s</v>
-      </c>
-      <c r="AW6" s="8" t="str">
-        <f t="shared" si="5"/>
-        <v>d</v>
-      </c>
-      <c r="AX6" s="8" t="str">
-        <f t="shared" si="5"/>
-        <v>l</v>
-      </c>
-      <c r="AY6" s="8" t="str">
-        <f t="shared" si="5"/>
-        <v>m</v>
-      </c>
-      <c r="AZ6" s="8" t="str">
-        <f t="shared" si="5"/>
-        <v>m</v>
-      </c>
-      <c r="BA6" s="8" t="str">
-        <f t="shared" si="5"/>
-        <v>j</v>
-      </c>
-      <c r="BB6" s="8" t="str">
-        <f t="shared" si="5"/>
-        <v>v</v>
-      </c>
-      <c r="BC6" s="8" t="str">
-        <f t="shared" si="5"/>
-        <v>s</v>
-      </c>
-      <c r="BD6" s="8" t="str">
-        <f t="shared" si="5"/>
-        <v>d</v>
-      </c>
-      <c r="BE6" s="8" t="str">
-        <f t="shared" si="5"/>
-        <v>l</v>
-      </c>
-      <c r="BF6" s="8" t="str">
-        <f t="shared" si="5"/>
-        <v>m</v>
-      </c>
-      <c r="BG6" s="8" t="str">
-        <f t="shared" si="5"/>
-        <v>m</v>
-      </c>
-      <c r="BH6" s="8" t="str">
-        <f t="shared" si="5"/>
-        <v>j</v>
-      </c>
-      <c r="BI6" s="8" t="str">
-        <f t="shared" si="5"/>
-        <v>v</v>
-      </c>
-      <c r="BJ6" s="8" t="str">
-        <f t="shared" si="5"/>
-        <v>s</v>
-      </c>
-      <c r="BK6" s="8" t="str">
-        <f t="shared" si="5"/>
-        <v>d</v>
-      </c>
     </row>
-    <row r="7" spans="1:63" ht="30" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:56" ht="30" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="25" t="s">
         <v>13</v>
       </c>
@@ -2533,15 +2428,8 @@
       <c r="BB7" s="22"/>
       <c r="BC7" s="22"/>
       <c r="BD7" s="22"/>
-      <c r="BE7" s="22"/>
-      <c r="BF7" s="22"/>
-      <c r="BG7" s="22"/>
-      <c r="BH7" s="22"/>
-      <c r="BI7" s="22"/>
-      <c r="BJ7" s="22"/>
-      <c r="BK7" s="22"/>
     </row>
-    <row r="8" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="26" t="s">
         <v>14</v>
       </c>
@@ -2553,7 +2441,7 @@
       <c r="E8" s="38"/>
       <c r="F8" s="9"/>
       <c r="G8" s="9" t="str">
-        <f t="shared" ref="G8:G41" si="6">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+        <f t="shared" ref="G8:G39" si="5">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v/>
       </c>
       <c r="H8" s="22"/>
@@ -2605,15 +2493,8 @@
       <c r="BB8" s="22"/>
       <c r="BC8" s="22"/>
       <c r="BD8" s="22"/>
-      <c r="BE8" s="64"/>
-      <c r="BF8" s="22"/>
-      <c r="BG8" s="22"/>
-      <c r="BH8" s="22"/>
-      <c r="BI8" s="22"/>
-      <c r="BJ8" s="22"/>
-      <c r="BK8" s="22"/>
     </row>
-    <row r="9" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="26" t="s">
         <v>15</v>
       </c>
@@ -2633,7 +2514,7 @@
       </c>
       <c r="F9" s="9"/>
       <c r="G9" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="H9" s="22"/>
@@ -2685,15 +2566,8 @@
       <c r="BB9" s="22"/>
       <c r="BC9" s="22"/>
       <c r="BD9" s="22"/>
-      <c r="BE9" s="22"/>
-      <c r="BF9" s="22"/>
-      <c r="BG9" s="22"/>
-      <c r="BH9" s="22"/>
-      <c r="BI9" s="22"/>
-      <c r="BJ9" s="22"/>
-      <c r="BK9" s="22"/>
     </row>
-    <row r="10" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="26" t="s">
         <v>16</v>
       </c>
@@ -2713,7 +2587,7 @@
       </c>
       <c r="F10" s="9"/>
       <c r="G10" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="H10" s="22"/>
@@ -2765,15 +2639,8 @@
       <c r="BB10" s="22"/>
       <c r="BC10" s="22"/>
       <c r="BD10" s="22"/>
-      <c r="BE10" s="22"/>
-      <c r="BF10" s="22"/>
-      <c r="BG10" s="22"/>
-      <c r="BH10" s="22"/>
-      <c r="BI10" s="22"/>
-      <c r="BJ10" s="22"/>
-      <c r="BK10" s="22"/>
     </row>
-    <row r="11" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="25"/>
       <c r="B11" s="30" t="s">
         <v>25</v>
@@ -2791,7 +2658,7 @@
       </c>
       <c r="F11" s="9"/>
       <c r="G11" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="H11" s="22"/>
@@ -2843,15 +2710,8 @@
       <c r="BB11" s="22"/>
       <c r="BC11" s="22"/>
       <c r="BD11" s="22"/>
-      <c r="BE11" s="22"/>
-      <c r="BF11" s="22"/>
-      <c r="BG11" s="22"/>
-      <c r="BH11" s="22"/>
-      <c r="BI11" s="22"/>
-      <c r="BJ11" s="22"/>
-      <c r="BK11" s="22"/>
     </row>
-    <row r="12" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="26" t="s">
         <v>17</v>
       </c>
@@ -2863,7 +2723,7 @@
       <c r="E12" s="41"/>
       <c r="F12" s="9"/>
       <c r="G12" s="9" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="H12" s="22"/>
@@ -2914,15 +2774,8 @@
       <c r="BB12" s="22"/>
       <c r="BC12" s="22"/>
       <c r="BD12" s="22"/>
-      <c r="BE12" s="22"/>
-      <c r="BF12" s="22"/>
-      <c r="BG12" s="22"/>
-      <c r="BH12" s="22"/>
-      <c r="BI12" s="22"/>
-      <c r="BJ12" s="22"/>
-      <c r="BK12" s="22"/>
     </row>
-    <row r="13" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="26"/>
       <c r="B13" s="31" t="s">
         <v>26</v>
@@ -2940,7 +2793,7 @@
       </c>
       <c r="F13" s="9"/>
       <c r="G13" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>2</v>
       </c>
       <c r="H13" s="22"/>
@@ -2992,15 +2845,8 @@
       <c r="BB13" s="22"/>
       <c r="BC13" s="22"/>
       <c r="BD13" s="22"/>
-      <c r="BE13" s="22"/>
-      <c r="BF13" s="22"/>
-      <c r="BG13" s="22"/>
-      <c r="BH13" s="22"/>
-      <c r="BI13" s="22"/>
-      <c r="BJ13" s="22"/>
-      <c r="BK13" s="22"/>
     </row>
-    <row r="14" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="25"/>
       <c r="B14" s="31" t="s">
         <v>27</v>
@@ -3009,7 +2855,7 @@
         <v>1</v>
       </c>
       <c r="D14" s="42">
-        <f t="shared" ref="D14:D30" si="7">E13+1</f>
+        <f t="shared" ref="D14:D30" si="6">E13+1</f>
         <v>46117</v>
       </c>
       <c r="E14" s="42">
@@ -3018,7 +2864,7 @@
       </c>
       <c r="F14" s="9"/>
       <c r="G14" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>2</v>
       </c>
       <c r="H14" s="22"/>
@@ -3070,15 +2916,8 @@
       <c r="BB14" s="22"/>
       <c r="BC14" s="22"/>
       <c r="BD14" s="22"/>
-      <c r="BE14" s="22"/>
-      <c r="BF14" s="22"/>
-      <c r="BG14" s="22"/>
-      <c r="BH14" s="22"/>
-      <c r="BI14" s="22"/>
-      <c r="BJ14" s="22"/>
-      <c r="BK14" s="22"/>
     </row>
-    <row r="15" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="25"/>
       <c r="B15" s="31" t="s">
         <v>28</v>
@@ -3087,7 +2926,7 @@
         <v>1</v>
       </c>
       <c r="D15" s="42">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>46119</v>
       </c>
       <c r="E15" s="42">
@@ -3096,7 +2935,7 @@
       </c>
       <c r="F15" s="9"/>
       <c r="G15" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="H15" s="22"/>
@@ -3148,15 +2987,8 @@
       <c r="BB15" s="22"/>
       <c r="BC15" s="22"/>
       <c r="BD15" s="22"/>
-      <c r="BE15" s="22"/>
-      <c r="BF15" s="22"/>
-      <c r="BG15" s="22"/>
-      <c r="BH15" s="22"/>
-      <c r="BI15" s="22"/>
-      <c r="BJ15" s="22"/>
-      <c r="BK15" s="22"/>
     </row>
-    <row r="16" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="25"/>
       <c r="B16" s="31" t="s">
         <v>30</v>
@@ -3174,7 +3006,7 @@
       </c>
       <c r="F16" s="9"/>
       <c r="G16" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="H16" s="22"/>
@@ -3226,15 +3058,8 @@
       <c r="BB16" s="22"/>
       <c r="BC16" s="22"/>
       <c r="BD16" s="22"/>
-      <c r="BE16" s="22"/>
-      <c r="BF16" s="22"/>
-      <c r="BG16" s="22"/>
-      <c r="BH16" s="22"/>
-      <c r="BI16" s="22"/>
-      <c r="BJ16" s="22"/>
-      <c r="BK16" s="22"/>
     </row>
-    <row r="17" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="25"/>
       <c r="B17" s="31" t="s">
         <v>29</v>
@@ -3243,7 +3068,7 @@
         <v>1</v>
       </c>
       <c r="D17" s="42">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>46120</v>
       </c>
       <c r="E17" s="42">
@@ -3252,7 +3077,7 @@
       </c>
       <c r="F17" s="9"/>
       <c r="G17" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="H17" s="22"/>
@@ -3304,18 +3129,11 @@
       <c r="BB17" s="22"/>
       <c r="BC17" s="22"/>
       <c r="BD17" s="22"/>
-      <c r="BE17" s="22"/>
-      <c r="BF17" s="22"/>
-      <c r="BG17" s="22"/>
-      <c r="BH17" s="22"/>
-      <c r="BI17" s="22"/>
-      <c r="BJ17" s="22"/>
-      <c r="BK17" s="22"/>
     </row>
-    <row r="18" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="25"/>
       <c r="B18" s="31" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C18" s="15">
         <v>1</v>
@@ -3379,15 +3197,8 @@
       <c r="BB18" s="22"/>
       <c r="BC18" s="22"/>
       <c r="BD18" s="22"/>
-      <c r="BE18" s="22"/>
-      <c r="BF18" s="22"/>
-      <c r="BG18" s="22"/>
-      <c r="BH18" s="22"/>
-      <c r="BI18" s="22"/>
-      <c r="BJ18" s="22"/>
-      <c r="BK18" s="22"/>
     </row>
-    <row r="19" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="25"/>
       <c r="B19" s="31" t="s">
         <v>31</v>
@@ -3405,7 +3216,7 @@
       </c>
       <c r="F19" s="9"/>
       <c r="G19" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>3</v>
       </c>
       <c r="H19" s="22"/>
@@ -3457,15 +3268,8 @@
       <c r="BB19" s="22"/>
       <c r="BC19" s="22"/>
       <c r="BD19" s="22"/>
-      <c r="BE19" s="22"/>
-      <c r="BF19" s="22"/>
-      <c r="BG19" s="22"/>
-      <c r="BH19" s="22"/>
-      <c r="BI19" s="22"/>
-      <c r="BJ19" s="22"/>
-      <c r="BK19" s="22"/>
     </row>
-    <row r="20" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="25"/>
       <c r="B20" s="31" t="s">
         <v>33</v>
@@ -3474,7 +3278,7 @@
         <v>1</v>
       </c>
       <c r="D20" s="42">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>46124</v>
       </c>
       <c r="E20" s="42">
@@ -3532,15 +3336,8 @@
       <c r="BB20" s="22"/>
       <c r="BC20" s="22"/>
       <c r="BD20" s="22"/>
-      <c r="BE20" s="22"/>
-      <c r="BF20" s="22"/>
-      <c r="BG20" s="22"/>
-      <c r="BH20" s="22"/>
-      <c r="BI20" s="22"/>
-      <c r="BJ20" s="22"/>
-      <c r="BK20" s="22"/>
     </row>
-    <row r="21" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="25"/>
       <c r="B21" s="31" t="s">
         <v>34</v>
@@ -3549,7 +3346,7 @@
         <v>1</v>
       </c>
       <c r="D21" s="42">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>46127</v>
       </c>
       <c r="E21" s="42">
@@ -3607,15 +3404,8 @@
       <c r="BB21" s="22"/>
       <c r="BC21" s="22"/>
       <c r="BD21" s="22"/>
-      <c r="BE21" s="22"/>
-      <c r="BF21" s="22"/>
-      <c r="BG21" s="22"/>
-      <c r="BH21" s="22"/>
-      <c r="BI21" s="22"/>
-      <c r="BJ21" s="22"/>
-      <c r="BK21" s="22"/>
     </row>
-    <row r="22" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="25"/>
       <c r="B22" s="31" t="s">
         <v>35</v>
@@ -3624,7 +3414,7 @@
         <v>1</v>
       </c>
       <c r="D22" s="42">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>46129</v>
       </c>
       <c r="E22" s="42">
@@ -3682,15 +3472,8 @@
       <c r="BB22" s="22"/>
       <c r="BC22" s="22"/>
       <c r="BD22" s="22"/>
-      <c r="BE22" s="22"/>
-      <c r="BF22" s="22"/>
-      <c r="BG22" s="22"/>
-      <c r="BH22" s="22"/>
-      <c r="BI22" s="22"/>
-      <c r="BJ22" s="22"/>
-      <c r="BK22" s="22"/>
     </row>
-    <row r="23" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="25"/>
       <c r="B23" s="31" t="s">
         <v>36</v>
@@ -3699,7 +3482,7 @@
         <v>1</v>
       </c>
       <c r="D23" s="42">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>46131</v>
       </c>
       <c r="E23" s="42">
@@ -3757,15 +3540,8 @@
       <c r="BB23" s="22"/>
       <c r="BC23" s="22"/>
       <c r="BD23" s="22"/>
-      <c r="BE23" s="22"/>
-      <c r="BF23" s="22"/>
-      <c r="BG23" s="22"/>
-      <c r="BH23" s="22"/>
-      <c r="BI23" s="22"/>
-      <c r="BJ23" s="22"/>
-      <c r="BK23" s="22"/>
     </row>
-    <row r="24" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="25"/>
       <c r="B24" s="31" t="s">
         <v>37</v>
@@ -3774,11 +3550,11 @@
         <v>1</v>
       </c>
       <c r="D24" s="42">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>46132</v>
       </c>
       <c r="E24" s="42">
-        <f t="shared" ref="E24:E29" si="8">D24+1</f>
+        <f t="shared" ref="E24:E29" si="7">D24+1</f>
         <v>46133</v>
       </c>
       <c r="F24" s="9"/>
@@ -3832,15 +3608,8 @@
       <c r="BB24" s="22"/>
       <c r="BC24" s="22"/>
       <c r="BD24" s="22"/>
-      <c r="BE24" s="22"/>
-      <c r="BF24" s="22"/>
-      <c r="BG24" s="22"/>
-      <c r="BH24" s="22"/>
-      <c r="BI24" s="22"/>
-      <c r="BJ24" s="22"/>
-      <c r="BK24" s="22"/>
     </row>
-    <row r="25" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="25"/>
       <c r="B25" s="31" t="s">
         <v>38</v>
@@ -3853,7 +3622,7 @@
         <v>46132</v>
       </c>
       <c r="E25" s="42">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>46133</v>
       </c>
       <c r="F25" s="9"/>
@@ -3907,15 +3676,8 @@
       <c r="BB25" s="22"/>
       <c r="BC25" s="22"/>
       <c r="BD25" s="22"/>
-      <c r="BE25" s="22"/>
-      <c r="BF25" s="22"/>
-      <c r="BG25" s="22"/>
-      <c r="BH25" s="22"/>
-      <c r="BI25" s="22"/>
-      <c r="BJ25" s="22"/>
-      <c r="BK25" s="22"/>
     </row>
-    <row r="26" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="25"/>
       <c r="B26" s="31" t="s">
         <v>39</v>
@@ -3924,11 +3686,11 @@
         <v>1</v>
       </c>
       <c r="D26" s="42">
+        <f t="shared" si="6"/>
+        <v>46134</v>
+      </c>
+      <c r="E26" s="42">
         <f t="shared" si="7"/>
-        <v>46134</v>
-      </c>
-      <c r="E26" s="42">
-        <f t="shared" si="8"/>
         <v>46135</v>
       </c>
       <c r="F26" s="9"/>
@@ -3982,18 +3744,11 @@
       <c r="BB26" s="22"/>
       <c r="BC26" s="22"/>
       <c r="BD26" s="22"/>
-      <c r="BE26" s="22"/>
-      <c r="BF26" s="22"/>
-      <c r="BG26" s="22"/>
-      <c r="BH26" s="22"/>
-      <c r="BI26" s="22"/>
-      <c r="BJ26" s="22"/>
-      <c r="BK26" s="22"/>
     </row>
-    <row r="27" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="25"/>
       <c r="B27" s="31" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C27" s="15">
         <v>1</v>
@@ -4003,7 +3758,7 @@
         <v>46136</v>
       </c>
       <c r="E27" s="42">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>46137</v>
       </c>
       <c r="F27" s="9"/>
@@ -4057,15 +3812,8 @@
       <c r="BB27" s="22"/>
       <c r="BC27" s="22"/>
       <c r="BD27" s="22"/>
-      <c r="BE27" s="22"/>
-      <c r="BF27" s="22"/>
-      <c r="BG27" s="22"/>
-      <c r="BH27" s="22"/>
-      <c r="BI27" s="22"/>
-      <c r="BJ27" s="22"/>
-      <c r="BK27" s="22"/>
     </row>
-    <row r="28" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="25"/>
       <c r="B28" s="31" t="s">
         <v>40</v>
@@ -4078,7 +3826,7 @@
         <v>46136</v>
       </c>
       <c r="E28" s="42">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>46137</v>
       </c>
       <c r="F28" s="9"/>
@@ -4132,15 +3880,8 @@
       <c r="BB28" s="22"/>
       <c r="BC28" s="22"/>
       <c r="BD28" s="22"/>
-      <c r="BE28" s="22"/>
-      <c r="BF28" s="22"/>
-      <c r="BG28" s="22"/>
-      <c r="BH28" s="22"/>
-      <c r="BI28" s="22"/>
-      <c r="BJ28" s="22"/>
-      <c r="BK28" s="22"/>
     </row>
-    <row r="29" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="25"/>
       <c r="B29" s="31" t="s">
         <v>41</v>
@@ -4153,7 +3894,7 @@
         <v>46138</v>
       </c>
       <c r="E29" s="42">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>46139</v>
       </c>
       <c r="F29" s="9"/>
@@ -4207,15 +3948,8 @@
       <c r="BB29" s="22"/>
       <c r="BC29" s="22"/>
       <c r="BD29" s="22"/>
-      <c r="BE29" s="22"/>
-      <c r="BF29" s="22"/>
-      <c r="BG29" s="22"/>
-      <c r="BH29" s="22"/>
-      <c r="BI29" s="22"/>
-      <c r="BJ29" s="22"/>
-      <c r="BK29" s="22"/>
     </row>
-    <row r="30" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="25"/>
       <c r="B30" s="31" t="s">
         <v>42</v>
@@ -4224,7 +3958,7 @@
         <v>1</v>
       </c>
       <c r="D30" s="42">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>46140</v>
       </c>
       <c r="E30" s="42">
@@ -4282,15 +4016,8 @@
       <c r="BB30" s="22"/>
       <c r="BC30" s="22"/>
       <c r="BD30" s="22"/>
-      <c r="BE30" s="22"/>
-      <c r="BF30" s="22"/>
-      <c r="BG30" s="22"/>
-      <c r="BH30" s="22"/>
-      <c r="BI30" s="22"/>
-      <c r="BJ30" s="22"/>
-      <c r="BK30" s="22"/>
     </row>
-    <row r="31" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="25" t="s">
         <v>18</v>
       </c>
@@ -4302,7 +4029,7 @@
       <c r="E31" s="44"/>
       <c r="F31" s="9"/>
       <c r="G31" s="9" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="H31" s="22"/>
@@ -4354,15 +4081,8 @@
       <c r="BB31" s="22"/>
       <c r="BC31" s="22"/>
       <c r="BD31" s="22"/>
-      <c r="BE31" s="22"/>
-      <c r="BF31" s="22"/>
-      <c r="BG31" s="22"/>
-      <c r="BH31" s="22"/>
-      <c r="BI31" s="22"/>
-      <c r="BJ31" s="22"/>
-      <c r="BK31" s="22"/>
     </row>
-    <row r="32" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="25"/>
       <c r="B32" s="32" t="s">
         <v>43</v>
@@ -4380,7 +4100,7 @@
       </c>
       <c r="F32" s="9"/>
       <c r="G32" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="H32" s="22"/>
@@ -4432,15 +4152,8 @@
       <c r="BB32" s="22"/>
       <c r="BC32" s="22"/>
       <c r="BD32" s="22"/>
-      <c r="BE32" s="22"/>
-      <c r="BF32" s="22"/>
-      <c r="BG32" s="22"/>
-      <c r="BH32" s="22"/>
-      <c r="BI32" s="22"/>
-      <c r="BJ32" s="22"/>
-      <c r="BK32" s="22"/>
     </row>
-    <row r="33" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="25" t="s">
         <v>18</v>
       </c>
@@ -4452,7 +4165,7 @@
       <c r="E33" s="47"/>
       <c r="F33" s="9"/>
       <c r="G33" s="9" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="H33" s="22"/>
@@ -4504,18 +4217,11 @@
       <c r="BB33" s="22"/>
       <c r="BC33" s="22"/>
       <c r="BD33" s="22"/>
-      <c r="BE33" s="22"/>
-      <c r="BF33" s="22"/>
-      <c r="BG33" s="22"/>
-      <c r="BH33" s="22"/>
-      <c r="BI33" s="22"/>
-      <c r="BJ33" s="22"/>
-      <c r="BK33" s="22"/>
     </row>
-    <row r="34" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="25"/>
       <c r="B34" s="33" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C34" s="21">
         <v>1</v>
@@ -4530,7 +4236,7 @@
       </c>
       <c r="F34" s="9"/>
       <c r="G34" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="H34" s="22"/>
@@ -4582,20 +4288,15 @@
       <c r="BB34" s="22"/>
       <c r="BC34" s="22"/>
       <c r="BD34" s="22"/>
-      <c r="BE34" s="22"/>
-      <c r="BF34" s="22"/>
-      <c r="BG34" s="22"/>
-      <c r="BH34" s="22"/>
-      <c r="BI34" s="22"/>
-      <c r="BJ34" s="22"/>
-      <c r="BK34" s="22"/>
     </row>
-    <row r="35" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="25"/>
       <c r="B35" s="33" t="s">
-        <v>53</v>
-      </c>
-      <c r="C35" s="21"/>
+        <v>50</v>
+      </c>
+      <c r="C35" s="21">
+        <v>1</v>
+      </c>
       <c r="D35" s="48">
         <f>E34+1</f>
         <v>46143</v>
@@ -4606,7 +4307,7 @@
       </c>
       <c r="F35" s="9"/>
       <c r="G35" s="9">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>3</v>
       </c>
       <c r="H35" s="22"/>
@@ -4658,32 +4359,27 @@
       <c r="BB35" s="22"/>
       <c r="BC35" s="22"/>
       <c r="BD35" s="22"/>
-      <c r="BE35" s="22"/>
-      <c r="BF35" s="22"/>
-      <c r="BG35" s="22"/>
-      <c r="BH35" s="22"/>
-      <c r="BI35" s="22"/>
-      <c r="BJ35" s="22"/>
-      <c r="BK35" s="22"/>
     </row>
-    <row r="36" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="25"/>
       <c r="B36" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="C36" s="21"/>
+      <c r="C36" s="21">
+        <v>1</v>
+      </c>
       <c r="D36" s="48">
         <f>E35+1</f>
         <v>46146</v>
       </c>
       <c r="E36" s="48">
-        <f>D36</f>
-        <v>46146</v>
+        <f>D36+1</f>
+        <v>46147</v>
       </c>
       <c r="F36" s="9"/>
       <c r="G36" s="9">
-        <f t="shared" si="6"/>
-        <v>1</v>
+        <f t="shared" si="5"/>
+        <v>2</v>
       </c>
       <c r="H36" s="22"/>
       <c r="I36" s="22"/>
@@ -4734,15 +4430,8 @@
       <c r="BB36" s="22"/>
       <c r="BC36" s="22"/>
       <c r="BD36" s="22"/>
-      <c r="BE36" s="22"/>
-      <c r="BF36" s="22"/>
-      <c r="BG36" s="22"/>
-      <c r="BH36" s="22"/>
-      <c r="BI36" s="22"/>
-      <c r="BJ36" s="22"/>
-      <c r="BK36" s="22"/>
     </row>
-    <row r="37" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="25"/>
       <c r="B37" s="57" t="s">
         <v>22</v>
@@ -4801,27 +4490,22 @@
       <c r="BB37" s="22"/>
       <c r="BC37" s="22"/>
       <c r="BD37" s="22"/>
-      <c r="BE37" s="22"/>
-      <c r="BF37" s="22"/>
-      <c r="BG37" s="22"/>
-      <c r="BH37" s="22"/>
-      <c r="BI37" s="22"/>
-      <c r="BJ37" s="22"/>
-      <c r="BK37" s="22"/>
     </row>
-    <row r="38" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="25"/>
       <c r="B38" s="62" t="s">
-        <v>46</v>
-      </c>
-      <c r="C38" s="61"/>
+        <v>51</v>
+      </c>
+      <c r="C38" s="61">
+        <v>0.25</v>
+      </c>
       <c r="D38" s="63">
         <f>E36+1</f>
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="E38" s="63">
-        <f>D38+1</f>
-        <v>46148</v>
+        <f>D38+4</f>
+        <v>46152</v>
       </c>
       <c r="F38" s="9"/>
       <c r="G38" s="9"/>
@@ -4874,30 +4558,28 @@
       <c r="BB38" s="22"/>
       <c r="BC38" s="22"/>
       <c r="BD38" s="22"/>
-      <c r="BE38" s="22"/>
-      <c r="BF38" s="22"/>
-      <c r="BG38" s="22"/>
-      <c r="BH38" s="22"/>
-      <c r="BI38" s="22"/>
-      <c r="BJ38" s="22"/>
-      <c r="BK38" s="22"/>
     </row>
-    <row r="39" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="25"/>
+    <row r="39" spans="1:56" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="25" t="s">
+        <v>18</v>
+      </c>
       <c r="B39" s="62" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C39" s="61"/>
       <c r="D39" s="63">
         <f>E38+1</f>
-        <v>46149</v>
+        <v>46153</v>
       </c>
       <c r="E39" s="63">
-        <f>D39+1</f>
-        <v>46150</v>
+        <f>D39+5</f>
+        <v>46158</v>
       </c>
       <c r="F39" s="9"/>
-      <c r="G39" s="9"/>
+      <c r="G39" s="9">
+        <f t="shared" si="5"/>
+        <v>6</v>
+      </c>
       <c r="H39" s="22"/>
       <c r="I39" s="22"/>
       <c r="J39" s="22"/>
@@ -4947,168 +4629,9 @@
       <c r="BB39" s="22"/>
       <c r="BC39" s="22"/>
       <c r="BD39" s="22"/>
-      <c r="BE39" s="22"/>
-      <c r="BF39" s="22"/>
-      <c r="BG39" s="22"/>
-      <c r="BH39" s="22"/>
-      <c r="BI39" s="22"/>
-      <c r="BJ39" s="22"/>
-      <c r="BK39" s="22"/>
-    </row>
-    <row r="40" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="25"/>
-      <c r="B40" s="62" t="s">
-        <v>48</v>
-      </c>
-      <c r="C40" s="61"/>
-      <c r="D40" s="63">
-        <f>E39+1</f>
-        <v>46151</v>
-      </c>
-      <c r="E40" s="63">
-        <f>D40+1</f>
-        <v>46152</v>
-      </c>
-      <c r="F40" s="9"/>
-      <c r="G40" s="9"/>
-      <c r="H40" s="22"/>
-      <c r="I40" s="22"/>
-      <c r="J40" s="22"/>
-      <c r="K40" s="22"/>
-      <c r="L40" s="22"/>
-      <c r="M40" s="22"/>
-      <c r="N40" s="22"/>
-      <c r="O40" s="22"/>
-      <c r="P40" s="22"/>
-      <c r="Q40" s="22"/>
-      <c r="R40" s="22"/>
-      <c r="S40" s="22"/>
-      <c r="T40" s="22"/>
-      <c r="U40" s="22"/>
-      <c r="V40" s="22"/>
-      <c r="W40" s="22"/>
-      <c r="X40" s="22"/>
-      <c r="Y40" s="22"/>
-      <c r="Z40" s="22"/>
-      <c r="AA40" s="22"/>
-      <c r="AB40" s="22"/>
-      <c r="AC40" s="22"/>
-      <c r="AD40" s="22"/>
-      <c r="AE40" s="22"/>
-      <c r="AF40" s="22"/>
-      <c r="AG40" s="22"/>
-      <c r="AH40" s="22"/>
-      <c r="AI40" s="22"/>
-      <c r="AJ40" s="22"/>
-      <c r="AK40" s="22"/>
-      <c r="AL40" s="22"/>
-      <c r="AM40" s="22"/>
-      <c r="AN40" s="22"/>
-      <c r="AO40" s="22"/>
-      <c r="AP40" s="22"/>
-      <c r="AQ40" s="22"/>
-      <c r="AR40" s="22"/>
-      <c r="AS40" s="22"/>
-      <c r="AT40" s="22"/>
-      <c r="AU40" s="22"/>
-      <c r="AV40" s="22"/>
-      <c r="AW40" s="22"/>
-      <c r="AX40" s="22"/>
-      <c r="AY40" s="22"/>
-      <c r="AZ40" s="22"/>
-      <c r="BA40" s="22"/>
-      <c r="BB40" s="22"/>
-      <c r="BC40" s="22"/>
-      <c r="BD40" s="22"/>
-      <c r="BE40" s="22"/>
-      <c r="BF40" s="22"/>
-      <c r="BG40" s="22"/>
-      <c r="BH40" s="22"/>
-      <c r="BI40" s="22"/>
-      <c r="BJ40" s="22"/>
-      <c r="BK40" s="22"/>
-    </row>
-    <row r="41" spans="1:63" s="2" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="25" t="s">
-        <v>18</v>
-      </c>
-      <c r="B41" s="62" t="s">
-        <v>49</v>
-      </c>
-      <c r="C41" s="61"/>
-      <c r="D41" s="63">
-        <f>E40+1</f>
-        <v>46153</v>
-      </c>
-      <c r="E41" s="63">
-        <f>D41+3</f>
-        <v>46156</v>
-      </c>
-      <c r="F41" s="9"/>
-      <c r="G41" s="9">
-        <f t="shared" si="6"/>
-        <v>4</v>
-      </c>
-      <c r="H41" s="22"/>
-      <c r="I41" s="22"/>
-      <c r="J41" s="22"/>
-      <c r="K41" s="22"/>
-      <c r="L41" s="22"/>
-      <c r="M41" s="22"/>
-      <c r="N41" s="22"/>
-      <c r="O41" s="22"/>
-      <c r="P41" s="22"/>
-      <c r="Q41" s="22"/>
-      <c r="R41" s="22"/>
-      <c r="S41" s="22"/>
-      <c r="T41" s="22"/>
-      <c r="U41" s="22"/>
-      <c r="V41" s="22"/>
-      <c r="W41" s="22"/>
-      <c r="X41" s="22"/>
-      <c r="Y41" s="22"/>
-      <c r="Z41" s="22"/>
-      <c r="AA41" s="22"/>
-      <c r="AB41" s="22"/>
-      <c r="AC41" s="22"/>
-      <c r="AD41" s="22"/>
-      <c r="AE41" s="22"/>
-      <c r="AF41" s="22"/>
-      <c r="AG41" s="22"/>
-      <c r="AH41" s="22"/>
-      <c r="AI41" s="22"/>
-      <c r="AJ41" s="22"/>
-      <c r="AK41" s="22"/>
-      <c r="AL41" s="22"/>
-      <c r="AM41" s="22"/>
-      <c r="AN41" s="22"/>
-      <c r="AO41" s="22"/>
-      <c r="AP41" s="22"/>
-      <c r="AQ41" s="22"/>
-      <c r="AR41" s="22"/>
-      <c r="AS41" s="22"/>
-      <c r="AT41" s="22"/>
-      <c r="AU41" s="22"/>
-      <c r="AV41" s="22"/>
-      <c r="AW41" s="22"/>
-      <c r="AX41" s="22"/>
-      <c r="AY41" s="22"/>
-      <c r="AZ41" s="22"/>
-      <c r="BA41" s="22"/>
-      <c r="BB41" s="22"/>
-      <c r="BC41" s="22"/>
-      <c r="BD41" s="22"/>
-      <c r="BE41" s="22"/>
-      <c r="BF41" s="22"/>
-      <c r="BG41" s="22"/>
-      <c r="BH41" s="22"/>
-      <c r="BI41" s="22"/>
-      <c r="BJ41" s="22"/>
-      <c r="BK41" s="22"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="BE4:BK4"/>
+  <mergeCells count="8">
     <mergeCell ref="D3:E3"/>
     <mergeCell ref="H4:N4"/>
     <mergeCell ref="O4:U4"/>
@@ -5118,7 +4641,7 @@
     <mergeCell ref="AQ4:AW4"/>
     <mergeCell ref="AX4:BD4"/>
   </mergeCells>
-  <conditionalFormatting sqref="C31:C34 C7:C18">
+  <conditionalFormatting sqref="C31:C34 C7:C18 C38">
     <cfRule type="dataBar" priority="43">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5132,16 +4655,16 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H5:BK10 H13:BK18 H12:L12 N12:BK12 H11:M11 O11:BK11 H31:BK40">
-    <cfRule type="expression" dxfId="11" priority="62">
+  <conditionalFormatting sqref="H12:L12 H11:M11 H5:BC10 N12:BC12 O11:BC11 H13:BC39">
+    <cfRule type="expression" dxfId="8" priority="62">
       <formula>AND(TODAY()&gt;=H$5,TODAY()&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H7:BK10 H13:BK18 H12:L12 N12:BK12 H11:M11 O11:BK11 H31:BK40">
-    <cfRule type="expression" dxfId="10" priority="56">
+  <conditionalFormatting sqref="H12:L12 H11:M11 H7:BC10 N12:BC12 O11:BC11 H13:BC39">
+    <cfRule type="expression" dxfId="7" priority="56">
       <formula>AND(task_start&lt;=H$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=H$5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="57" stopIfTrue="1">
+    <cfRule type="expression" dxfId="6" priority="57" stopIfTrue="1">
       <formula>AND(task_end&gt;=H$5,task_start&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5157,19 +4680,6 @@
           <x14:id>{1E90BFA6-AA09-4C84-9DA7-1419DF975915}</x14:id>
         </ext>
       </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H19:BK30">
-    <cfRule type="expression" dxfId="8" priority="29">
-      <formula>AND(TODAY()&gt;=H$5,TODAY()&lt;I$5)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H19:BK30">
-    <cfRule type="expression" dxfId="7" priority="27">
-      <formula>AND(task_start&lt;=H$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=H$5)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="6" priority="28" stopIfTrue="1">
-      <formula>AND(task_end&gt;=H$5,task_start&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C21">
@@ -5326,7 +4836,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C41">
+  <conditionalFormatting sqref="C39">
     <cfRule type="dataBar" priority="3">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5338,19 +4848,6 @@
           <x14:id>{4BA551C2-EE6C-4479-BB90-42C647FFB418}</x14:id>
         </ext>
       </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H41:BK41">
-    <cfRule type="expression" dxfId="5" priority="6">
-      <formula>AND(TODAY()&gt;=H$5,TODAY()&lt;I$5)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H41:BK41">
-    <cfRule type="expression" dxfId="4" priority="4">
-      <formula>AND(task_start&lt;=H$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=H$5)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="3" priority="5" stopIfTrue="1">
-      <formula>AND(task_end&gt;=H$5,task_start&lt;I$5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C37">
@@ -5367,31 +4864,30 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C38:C40">
-    <cfRule type="dataBar" priority="1">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color theme="0" tint="-0.249977111117893"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{527A852E-2EF7-46F3-8CBA-90E4DD67FCB3}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="N11">
-    <cfRule type="expression" dxfId="2" priority="64">
+    <cfRule type="expression" dxfId="5" priority="64">
       <formula>AND(TODAY()&gt;=M$5,TODAY()&lt;N$5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N11">
-    <cfRule type="expression" dxfId="1" priority="67">
+    <cfRule type="expression" dxfId="4" priority="67">
       <formula>AND(task_start&lt;=M$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=M$5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="68" stopIfTrue="1">
+    <cfRule type="expression" dxfId="3" priority="68" stopIfTrue="1">
       <formula>AND(task_end&gt;=M$5,task_start&lt;N$5)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="BD5:BD39">
+    <cfRule type="expression" dxfId="2" priority="70">
+      <formula>AND(TODAY()&gt;=BD$5,TODAY()&lt;#REF!)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="BD7:BD39">
+    <cfRule type="expression" dxfId="1" priority="81">
+      <formula>AND(task_start&lt;=BD$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=BD$5)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="82" stopIfTrue="1">
+      <formula>AND(task_end&gt;=BD$5,task_start&lt;#REF!)</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -5401,7 +4897,7 @@
   </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.35" right="0.35" top="0.35" bottom="0.5" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="51" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="42" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <headerFooter differentFirst="1" scaleWithDoc="0">
     <oddFooter>Page &amp;P of &amp;N</oddFooter>
   </headerFooter>
@@ -5421,7 +4917,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>C31:C34 C7:C18</xm:sqref>
+          <xm:sqref>C31:C34 C7:C18 C38</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{1E90BFA6-AA09-4C84-9DA7-1419DF975915}">
@@ -5616,7 +5112,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>C41</xm:sqref>
+          <xm:sqref>C39</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{06F74896-8DFF-43FC-B666-14565B6A7397}">
@@ -5633,21 +5129,6 @@
           </x14:cfRule>
           <xm:sqref>C37</xm:sqref>
         </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{527A852E-2EF7-46F3-8CBA-90E4DD67FCB3}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>1</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>C38:C40</xm:sqref>
-        </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
   </extLst>
@@ -5655,35 +5136,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Image>
-    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
-    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </ImageTagsTaxHTField>
-    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
-    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="24" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2d714a3296df14eba7a100bb665443ca">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="49549bf45bfbbfb6cffed527380e77e1" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -5971,34 +5423,36 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5144944C-1F1D-4162-962A-96F3FC8455D8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="16c05727-aa75-4e4a-9b5f-8a80a1165891"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8FE8ED85-58B3-4608-8E91-0433556D50CE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Image>
+    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
+    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </ImageTagsTaxHTField>
+    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
+    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{708DBB9E-6D89-4A94-9DC5-964B7833E11C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6017,4 +5471,31 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8FE8ED85-58B3-4608-8E91-0433556D50CE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5144944C-1F1D-4162-962A-96F3FC8455D8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
+    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="16c05727-aa75-4e4a-9b5f-8a80a1165891"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>